<commit_message>
Atualização automática do relatório BI
</commit_message>
<xml_diff>
--- a/Relatório Construção.xlsx
+++ b/Relatório Construção.xlsx
@@ -844,7 +844,7 @@
         <v>45817.43766342592</v>
       </c>
       <c r="AW2">
-        <v>273.834282</v>
+        <v>274.834282</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -1022,7 +1022,7 @@
         <v>45974.32166768519</v>
       </c>
       <c r="AW3">
-        <v>116.950278</v>
+        <v>117.950278</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
@@ -1203,7 +1203,7 @@
         <v>45986.56362434028</v>
       </c>
       <c r="AW4">
-        <v>104.708322</v>
+        <v>105.708322</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -1379,7 +1379,7 @@
         <v>45862.49200517361</v>
       </c>
       <c r="AW5">
-        <v>228.779942</v>
+        <v>229.779942</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -1557,7 +1557,7 @@
         <v>45859.70545487269</v>
       </c>
       <c r="AW6">
-        <v>231.566493</v>
+        <v>232.566493</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -1738,7 +1738,7 @@
         <v>46051.33790607639</v>
       </c>
       <c r="AW7">
-        <v>39.934039</v>
+        <v>40.934039</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -1916,7 +1916,7 @@
         <v>45824.66795922453</v>
       </c>
       <c r="AW8">
-        <v>266.603993</v>
+        <v>267.603993</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -2100,7 +2100,7 @@
         <v>45875.62732515046</v>
       </c>
       <c r="AW9">
-        <v>215.64463</v>
+        <v>216.64463</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -2278,7 +2278,7 @@
         <v>45891.54403121528</v>
       </c>
       <c r="AW10">
-        <v>199.727917</v>
+        <v>200.727917</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -2459,7 +2459,7 @@
         <v>45975.64739481482</v>
       </c>
       <c r="AW11">
-        <v>115.62456</v>
+        <v>116.62456</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -2640,7 +2640,7 @@
         <v>45890.64166144676</v>
       </c>
       <c r="AW12">
-        <v>200.630289</v>
+        <v>201.630289</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -2818,7 +2818,7 @@
         <v>45812.58396733797</v>
       </c>
       <c r="AW13">
-        <v>278.687986</v>
+        <v>279.687986</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -2996,7 +2996,7 @@
         <v>45826.76881550926</v>
       </c>
       <c r="AW14">
-        <v>264.503137</v>
+        <v>265.503137</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -3174,7 +3174,7 @@
         <v>45856.44733234953</v>
       </c>
       <c r="AW15">
-        <v>233.631667</v>
+        <v>234.631667</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -3355,7 +3355,7 @@
         <v>45855.34298560185</v>
       </c>
       <c r="AW16">
-        <v>235.92897</v>
+        <v>236.92897</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -3536,7 +3536,7 @@
         <v>45975.69316193287</v>
       </c>
       <c r="AW17">
-        <v>115.578785</v>
+        <v>116.578785</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -3712,7 +3712,7 @@
         <v>45993.45690386574</v>
       </c>
       <c r="AW18">
-        <v>97.815046</v>
+        <v>98.815046</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -3893,7 +3893,7 @@
         <v>45887.7561505787</v>
       </c>
       <c r="AW19">
-        <v>203.515799</v>
+        <v>204.515799</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -4074,7 +4074,7 @@
         <v>45895.66738841435</v>
       </c>
       <c r="AW20">
-        <v>195.60456</v>
+        <v>196.60456</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -4255,7 +4255,7 @@
         <v>45974.32124640046</v>
       </c>
       <c r="AW21">
-        <v>116.950706</v>
+        <v>117.950706</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -4433,7 +4433,7 @@
         <v>46057.3192221875</v>
       </c>
       <c r="AW22">
-        <v>33.952731</v>
+        <v>34.952731</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -4614,7 +4614,7 @@
         <v>46058.5740270949</v>
       </c>
       <c r="AW23">
-        <v>32.697928</v>
+        <v>33.697928</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -4795,7 +4795,7 @@
         <v>46051.34049207176</v>
       </c>
       <c r="AW24">
-        <v>39.931458</v>
+        <v>40.931458</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -4971,7 +4971,7 @@
         <v>45862.49253582176</v>
       </c>
       <c r="AW25">
-        <v>228.77941</v>
+        <v>229.77941</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -5152,7 +5152,7 @@
         <v>45975.54832606482</v>
       </c>
       <c r="AW26">
-        <v>115.723623</v>
+        <v>116.723623</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -5330,7 +5330,7 @@
         <v>46077.69417114583</v>
       </c>
       <c r="AW27">
-        <v>13.577778</v>
+        <v>14.577778</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -5511,7 +5511,7 @@
         <v>46027.33752056713</v>
       </c>
       <c r="AW28">
-        <v>63.934433</v>
+        <v>64.934433</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -5697,7 +5697,7 @@
         <v>45826.76330768519</v>
       </c>
       <c r="AW29">
-        <v>264.508646</v>
+        <v>265.508646</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
@@ -5875,7 +5875,7 @@
         <v>45905.67982599537</v>
       </c>
       <c r="AW30">
-        <v>185.59213</v>
+        <v>186.59213</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -6056,7 +6056,7 @@
         <v>45896.58634196759</v>
       </c>
       <c r="AW31">
-        <v>194.685613</v>
+        <v>195.685613</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
@@ -6237,7 +6237,7 @@
         <v>45966.44628628472</v>
       </c>
       <c r="AW32">
-        <v>124.82566</v>
+        <v>125.82566</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -6415,7 +6415,7 @@
         <v>45824.67305528936</v>
       </c>
       <c r="AW33">
-        <v>266.5989</v>
+        <v>267.5989</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -6596,7 +6596,7 @@
         <v>45967.66489237269</v>
       </c>
       <c r="AW34">
-        <v>123.60706</v>
+        <v>124.60706</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
@@ -6777,7 +6777,7 @@
         <v>45888.44432909723</v>
       </c>
       <c r="AW35">
-        <v>202.827616</v>
+        <v>203.827616</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -6958,7 +6958,7 @@
         <v>45979.54654831019</v>
       </c>
       <c r="AW36">
-        <v>111.725405</v>
+        <v>112.725405</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
@@ -7136,7 +7136,7 @@
         <v>45860.39854054398</v>
       </c>
       <c r="AW37">
-        <v>230.873414</v>
+        <v>231.873414</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
@@ -7317,7 +7317,7 @@
         <v>45820.33365524306</v>
       </c>
       <c r="AW38">
-        <v>238.659155</v>
+        <v>239.659155</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
@@ -7451,7 +7451,7 @@
         <v>46090.58235540509</v>
       </c>
       <c r="AQ39">
-        <v>0.689595</v>
+        <v>1.689595</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
@@ -7632,7 +7632,7 @@
         <v>45965.38089574075</v>
       </c>
       <c r="AW40">
-        <v>125.891053</v>
+        <v>126.891053</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
@@ -7813,7 +7813,7 @@
         <v>45986.56665260416</v>
       </c>
       <c r="AW41">
-        <v>104.705301</v>
+        <v>105.705301</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
@@ -7994,7 +7994,7 @@
         <v>46027.57691234954</v>
       </c>
       <c r="AW42">
-        <v>63.695035</v>
+        <v>64.695035</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
@@ -8172,7 +8172,7 @@
         <v>46057.31722791667</v>
       </c>
       <c r="AW43">
-        <v>33.954722</v>
+        <v>34.954722</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
@@ -8353,7 +8353,7 @@
         <v>46037.65326952546</v>
       </c>
       <c r="AW44">
-        <v>53.618681</v>
+        <v>54.618681</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
@@ -8534,7 +8534,7 @@
         <v>46078.55323623843</v>
       </c>
       <c r="AW45">
-        <v>12.718715</v>
+        <v>13.718715</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
@@ -8715,7 +8715,7 @@
         <v>45903.36153759259</v>
       </c>
       <c r="AW46">
-        <v>187.910417</v>
+        <v>188.910417</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
@@ -8896,7 +8896,7 @@
         <v>45888.44494424769</v>
       </c>
       <c r="AW47">
-        <v>202.827002</v>
+        <v>203.827002</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
@@ -9030,7 +9030,7 @@
         <v>46090.58140600695</v>
       </c>
       <c r="AQ48">
-        <v>0.690544</v>
+        <v>1.690544</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
@@ -9214,7 +9214,7 @@
         <v>45924.33465340278</v>
       </c>
       <c r="AW49">
-        <v>153.943773</v>
+        <v>154.943773</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
@@ -9395,7 +9395,7 @@
         <v>45937.3293883912</v>
       </c>
       <c r="AW50">
-        <v>153.942558</v>
+        <v>154.942558</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -9563,7 +9563,7 @@
         <v>46079.67913538194</v>
       </c>
       <c r="AW51">
-        <v>11.592813</v>
+        <v>12.592813</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -9744,7 +9744,7 @@
         <v>45860.39754922454</v>
       </c>
       <c r="AW52">
-        <v>230.874398</v>
+        <v>231.874398</v>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
@@ -9922,7 +9922,7 @@
         <v>45859.70404015046</v>
       </c>
       <c r="AW53">
-        <v>231.567905</v>
+        <v>232.567905</v>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
@@ -10106,7 +10106,7 @@
         <v>45946.6547500926</v>
       </c>
       <c r="AW54">
-        <v>138.710521</v>
+        <v>139.710521</v>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
@@ -10287,7 +10287,7 @@
         <v>45846.48855997685</v>
       </c>
       <c r="AW55">
-        <v>244.783391</v>
+        <v>245.783391</v>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
@@ -10465,7 +10465,7 @@
         <v>46079.67988275463</v>
       </c>
       <c r="AW56">
-        <v>11.592072</v>
+        <v>12.592072</v>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
@@ -10649,7 +10649,7 @@
         <v>45868.73102224537</v>
       </c>
       <c r="AW57">
-        <v>222.540926</v>
+        <v>223.540926</v>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
@@ -10783,7 +10783,7 @@
         <v>46090.58088335648</v>
       </c>
       <c r="AQ58">
-        <v>0.691065</v>
+        <v>1.691065</v>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
@@ -10961,7 +10961,7 @@
         <v>45821.6263675</v>
       </c>
       <c r="AW59">
-        <v>269.645579</v>
+        <v>270.645579</v>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
@@ -11139,7 +11139,7 @@
         <v>45831.57755690972</v>
       </c>
       <c r="AW60">
-        <v>259.694398</v>
+        <v>260.694398</v>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
@@ -11320,7 +11320,7 @@
         <v>46001.47500929398</v>
       </c>
       <c r="AW61">
-        <v>89.796944</v>
+        <v>90.796944</v>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
@@ -11498,7 +11498,7 @@
         <v>46036.58371895833</v>
       </c>
       <c r="AW62">
-        <v>54.688229</v>
+        <v>55.688229</v>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
@@ -11676,7 +11676,7 @@
         <v>45859.70488313658</v>
       </c>
       <c r="AW63">
-        <v>231.567072</v>
+        <v>232.567072</v>
       </c>
     </row>
     <row r="64" ht="18" customHeight="1">
@@ -11857,7 +11857,7 @@
         <v>45965.37678740741</v>
       </c>
       <c r="AW64">
-        <v>125.895162</v>
+        <v>126.895162</v>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
@@ -12038,7 +12038,7 @@
         <v>45985.75714297454</v>
       </c>
       <c r="AW65">
-        <v>105.514803</v>
+        <v>106.514803</v>
       </c>
     </row>
     <row r="66" ht="18" customHeight="1">
@@ -12219,7 +12219,7 @@
         <v>45923.70330438657</v>
       </c>
       <c r="AW66">
-        <v>167.568646</v>
+        <v>168.568646</v>
       </c>
     </row>
     <row r="67" ht="18" customHeight="1">
@@ -12397,7 +12397,7 @@
         <v>45856.44919015047</v>
       </c>
       <c r="AW67">
-        <v>234.822755</v>
+        <v>235.822755</v>
       </c>
     </row>
     <row r="68" ht="18" customHeight="1">
@@ -12575,7 +12575,7 @@
         <v>45895.64805509259</v>
       </c>
       <c r="AW68">
-        <v>195.6239</v>
+        <v>196.6239</v>
       </c>
     </row>
     <row r="69" ht="18" customHeight="1">
@@ -12759,7 +12759,7 @@
         <v>45975.64818255787</v>
       </c>
       <c r="AW69">
-        <v>115.623773</v>
+        <v>116.623773</v>
       </c>
     </row>
     <row r="70" ht="18" customHeight="1">
@@ -12937,7 +12937,7 @@
         <v>46037.67363424769</v>
       </c>
       <c r="AW70">
-        <v>53.598322</v>
+        <v>54.598322</v>
       </c>
     </row>
     <row r="71" ht="18" customHeight="1">
@@ -13115,7 +13115,7 @@
         <v>45820.33324042824</v>
       </c>
       <c r="AW71">
-        <v>270.938715</v>
+        <v>271.938715</v>
       </c>
     </row>
     <row r="72" ht="18" customHeight="1">
@@ -13293,7 +13293,7 @@
         <v>45817.44034118055</v>
       </c>
       <c r="AW72">
-        <v>273.831609</v>
+        <v>274.831609</v>
       </c>
     </row>
     <row r="73" ht="18" customHeight="1">
@@ -13471,7 +13471,7 @@
         <v>45859.68910778935</v>
       </c>
       <c r="AW73">
-        <v>231.582847</v>
+        <v>232.582847</v>
       </c>
     </row>
     <row r="74" ht="18" customHeight="1">
@@ -13652,7 +13652,7 @@
         <v>45902.58757359954</v>
       </c>
       <c r="AW74">
-        <v>188.684375</v>
+        <v>189.684375</v>
       </c>
     </row>
     <row r="75" ht="18" customHeight="1">
@@ -13830,7 +13830,7 @@
         <v>45966.55098307871</v>
       </c>
       <c r="AW75">
-        <v>124.720972</v>
+        <v>125.720972</v>
       </c>
     </row>
     <row r="76" ht="18" customHeight="1">
@@ -14011,7 +14011,7 @@
         <v>45959.55501203703</v>
       </c>
       <c r="AW76">
-        <v>131.716933</v>
+        <v>132.716933</v>
       </c>
     </row>
     <row r="77" ht="18" customHeight="1">
@@ -14192,7 +14192,7 @@
         <v>46007.42731981481</v>
       </c>
       <c r="AW77">
-        <v>83.84463</v>
+        <v>84.84463</v>
       </c>
     </row>
     <row r="78" ht="18" customHeight="1">
@@ -14373,7 +14373,7 @@
         <v>46002.72977564814</v>
       </c>
       <c r="AW78">
-        <v>88.542176</v>
+        <v>89.542176</v>
       </c>
     </row>
     <row r="79" ht="18" customHeight="1">
@@ -14554,7 +14554,7 @@
         <v>46057.49838530092</v>
       </c>
       <c r="AW79">
-        <v>33.773565</v>
+        <v>34.773565</v>
       </c>
     </row>
     <row r="80" ht="18" customHeight="1">
@@ -14696,7 +14696,7 @@
         <v>46076.53149964121</v>
       </c>
       <c r="AQ80">
-        <v>14.740451</v>
+        <v>15.740451</v>
       </c>
     </row>
     <row r="81" ht="18" customHeight="1">
@@ -14882,7 +14882,7 @@
         <v>45845.61766498843</v>
       </c>
       <c r="AW81">
-        <v>245.654282</v>
+        <v>246.654282</v>
       </c>
     </row>
     <row r="82" ht="18" customHeight="1">
@@ -15060,7 +15060,7 @@
         <v>45908.5914516551</v>
       </c>
       <c r="AW82">
-        <v>182.680498</v>
+        <v>183.680498</v>
       </c>
     </row>
     <row r="83" ht="18" customHeight="1">
@@ -15241,7 +15241,7 @@
         <v>45973.66445978009</v>
       </c>
       <c r="AW83">
-        <v>117.607488</v>
+        <v>118.607488</v>
       </c>
     </row>
     <row r="84" ht="18" customHeight="1">
@@ -15378,7 +15378,7 @@
         <v>46090.72432047454</v>
       </c>
       <c r="AQ84">
-        <v>0.547627</v>
+        <v>1.547627</v>
       </c>
     </row>
     <row r="85" ht="18" customHeight="1">
@@ -15562,7 +15562,7 @@
         <v>45894.4102940162</v>
       </c>
       <c r="AW85">
-        <v>186.889144</v>
+        <v>187.889144</v>
       </c>
     </row>
     <row r="86" ht="18" customHeight="1">
@@ -15743,7 +15743,7 @@
         <v>45986.57630509259</v>
       </c>
       <c r="AW86">
-        <v>104.695648</v>
+        <v>105.695648</v>
       </c>
     </row>
     <row r="87" ht="18" customHeight="1">
@@ -15924,7 +15924,7 @@
         <v>45831.57415840278</v>
       </c>
       <c r="AW87">
-        <v>259.697789</v>
+        <v>260.697789</v>
       </c>
     </row>
     <row r="88" ht="18" customHeight="1">
@@ -16105,7 +16105,7 @@
         <v>45937.3283994213</v>
       </c>
       <c r="AW88">
-        <v>153.943553</v>
+        <v>154.943553</v>
       </c>
     </row>
     <row r="89" ht="18" customHeight="1">
@@ -16283,7 +16283,7 @@
         <v>45952.41303611111</v>
       </c>
       <c r="AW89">
-        <v>138.858912</v>
+        <v>139.858912</v>
       </c>
     </row>
     <row r="90" ht="18" customHeight="1">
@@ -16464,7 +16464,7 @@
         <v>45957.71828232639</v>
       </c>
       <c r="AW90">
-        <v>133.553669</v>
+        <v>134.553669</v>
       </c>
     </row>
     <row r="91" ht="18" customHeight="1">
@@ -16645,7 +16645,7 @@
         <v>45967.6662366088</v>
       </c>
       <c r="AW91">
-        <v>123.605718</v>
+        <v>124.605718</v>
       </c>
     </row>
     <row r="92" ht="18" customHeight="1">
@@ -16823,7 +16823,7 @@
         <v>45852.54883409722</v>
       </c>
       <c r="AW92">
-        <v>238.723113</v>
+        <v>239.723113</v>
       </c>
     </row>
     <row r="93" ht="18" customHeight="1">
@@ -17001,7 +17001,7 @@
         <v>45821.67408983796</v>
       </c>
       <c r="AW93">
-        <v>269.597859</v>
+        <v>270.597859</v>
       </c>
     </row>
     <row r="94" ht="18" customHeight="1">
@@ -17190,7 +17190,7 @@
         <v>45873.70541589121</v>
       </c>
       <c r="AW94">
-        <v>217.567523</v>
+        <v>218.567523</v>
       </c>
     </row>
     <row r="95" ht="18" customHeight="1">
@@ -17371,7 +17371,7 @@
         <v>45904.38451509259</v>
       </c>
       <c r="AW95">
-        <v>186.887431</v>
+        <v>187.887431</v>
       </c>
     </row>
     <row r="96" ht="18" customHeight="1">
@@ -17552,7 +17552,7 @@
         <v>45923.7104591088</v>
       </c>
       <c r="AW96">
-        <v>167.561493</v>
+        <v>168.561493</v>
       </c>
     </row>
     <row r="97" ht="18" customHeight="1">
@@ -17733,7 +17733,7 @@
         <v>46001.46563837962</v>
       </c>
       <c r="AW97">
-        <v>89.806308</v>
+        <v>90.806308</v>
       </c>
     </row>
     <row r="98" ht="18" customHeight="1">
@@ -17834,7 +17834,7 @@
         <v>46076.60414643519</v>
       </c>
       <c r="AK98">
-        <v>14.667801</v>
+        <v>15.667801</v>
       </c>
     </row>
     <row r="99" ht="18" customHeight="1">
@@ -18015,7 +18015,7 @@
         <v>45817.66125234954</v>
       </c>
       <c r="AW99">
-        <v>223.570035</v>
+        <v>224.570035</v>
       </c>
     </row>
     <row r="100" ht="18" customHeight="1">
@@ -18193,7 +18193,7 @@
         <v>45826.76919975695</v>
       </c>
       <c r="AW100">
-        <v>264.502755</v>
+        <v>265.502755</v>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1">
@@ -18371,7 +18371,7 @@
         <v>45917.32877043981</v>
       </c>
       <c r="AW101">
-        <v>173.943183</v>
+        <v>174.943183</v>
       </c>
     </row>
     <row r="102" ht="18" customHeight="1">
@@ -18549,7 +18549,7 @@
         <v>45859.7056584838</v>
       </c>
       <c r="AW102">
-        <v>231.566296</v>
+        <v>232.566296</v>
       </c>
     </row>
     <row r="103" ht="18" customHeight="1">
@@ -18730,7 +18730,7 @@
         <v>46027.3338925</v>
       </c>
       <c r="AW103">
-        <v>63.938056</v>
+        <v>64.938056</v>
       </c>
     </row>
     <row r="104" ht="18" customHeight="1">
@@ -18908,7 +18908,7 @@
         <v>45820.33284418982</v>
       </c>
       <c r="AW104">
-        <v>270.939109</v>
+        <v>271.939109</v>
       </c>
     </row>
     <row r="105" ht="18" customHeight="1">
@@ -19086,7 +19086,7 @@
         <v>45908.71817314815</v>
       </c>
       <c r="AW105">
-        <v>182.553773</v>
+        <v>183.553773</v>
       </c>
     </row>
     <row r="106" ht="18" customHeight="1">
@@ -19267,7 +19267,7 @@
         <v>45986.56307221065</v>
       </c>
       <c r="AW106">
-        <v>104.708877</v>
+        <v>105.708877</v>
       </c>
     </row>
     <row r="107" ht="18" customHeight="1">
@@ -19448,7 +19448,7 @@
         <v>45890.64899726852</v>
       </c>
       <c r="AW107">
-        <v>200.622951</v>
+        <v>201.622951</v>
       </c>
     </row>
     <row r="108" ht="18" customHeight="1">
@@ -19629,7 +19629,7 @@
         <v>45898.57314238426</v>
       </c>
       <c r="AW108">
-        <v>192.698808</v>
+        <v>193.698808</v>
       </c>
     </row>
     <row r="109" ht="18" customHeight="1">
@@ -19807,7 +19807,7 @@
         <v>46058.54936295139</v>
       </c>
       <c r="AW109">
-        <v>32.722593</v>
+        <v>33.722593</v>
       </c>
     </row>
     <row r="110" ht="18" customHeight="1">
@@ -19985,7 +19985,7 @@
         <v>45824.58323728009</v>
       </c>
       <c r="AW110">
-        <v>266.688715</v>
+        <v>267.688715</v>
       </c>
     </row>
     <row r="111" ht="18" customHeight="1">
@@ -20166,7 +20166,7 @@
         <v>45868.58624710648</v>
       </c>
       <c r="AW111">
-        <v>222.685706</v>
+        <v>223.685706</v>
       </c>
     </row>
     <row r="112" ht="18" customHeight="1">
@@ -20350,7 +20350,7 @@
         <v>45875.68373804398</v>
       </c>
       <c r="AW112">
-        <v>161.944456</v>
+        <v>162.944456</v>
       </c>
     </row>
     <row r="113" ht="18" customHeight="1">
@@ -20531,7 +20531,7 @@
         <v>45987.54818097223</v>
       </c>
       <c r="AW113">
-        <v>103.723773</v>
+        <v>104.723773</v>
       </c>
     </row>
     <row r="114" ht="18" customHeight="1">
@@ -20712,7 +20712,7 @@
         <v>45817.43553984954</v>
       </c>
       <c r="AW114">
-        <v>221.122581</v>
+        <v>222.122581</v>
       </c>
     </row>
     <row r="115" ht="18" customHeight="1">
@@ -20893,7 +20893,7 @@
         <v>45861.50585359953</v>
       </c>
       <c r="AW115">
-        <v>229.7661</v>
+        <v>230.7661</v>
       </c>
     </row>
     <row r="116" ht="18" customHeight="1">
@@ -21074,7 +21074,7 @@
         <v>45908.66222837963</v>
       </c>
       <c r="AW116">
-        <v>182.609722</v>
+        <v>183.609722</v>
       </c>
     </row>
     <row r="117" ht="18" customHeight="1">
@@ -21255,7 +21255,7 @@
         <v>45959.57354159722</v>
       </c>
       <c r="AW117">
-        <v>131.698414</v>
+        <v>132.698414</v>
       </c>
     </row>
     <row r="118" ht="18" customHeight="1">
@@ -21436,7 +21436,7 @@
         <v>45986.5776178125</v>
       </c>
       <c r="AW118">
-        <v>104.694329</v>
+        <v>105.694329</v>
       </c>
     </row>
     <row r="119" ht="18" customHeight="1">
@@ -21617,7 +21617,7 @@
         <v>46027.33527493056</v>
       </c>
       <c r="AW119">
-        <v>63.936678</v>
+        <v>64.936678</v>
       </c>
     </row>
     <row r="120" ht="18" customHeight="1">
@@ -21798,7 +21798,7 @@
         <v>46050.54798530092</v>
       </c>
       <c r="AW120">
-        <v>40.72397</v>
+        <v>41.72397</v>
       </c>
     </row>
     <row r="121" ht="18" customHeight="1">
@@ -21976,7 +21976,7 @@
         <v>45817.43738373843</v>
       </c>
       <c r="AW121">
-        <v>273.834572</v>
+        <v>274.834572</v>
       </c>
     </row>
     <row r="122" ht="18" customHeight="1">
@@ -22154,7 +22154,7 @@
         <v>45831.62649351852</v>
       </c>
       <c r="AW122">
-        <v>259.645451</v>
+        <v>260.645451</v>
       </c>
     </row>
     <row r="123" ht="18" customHeight="1">
@@ -22335,7 +22335,7 @@
         <v>45821.67595234954</v>
       </c>
       <c r="AW123">
-        <v>269.595995</v>
+        <v>270.595995</v>
       </c>
     </row>
     <row r="124" ht="18" customHeight="1">
@@ -22516,7 +22516,7 @@
         <v>45929.32908571759</v>
       </c>
       <c r="AW124">
-        <v>161.942859</v>
+        <v>162.942859</v>
       </c>
     </row>
     <row r="125" ht="18" customHeight="1">
@@ -22697,7 +22697,7 @@
         <v>45975.54881452546</v>
       </c>
       <c r="AW125">
-        <v>115.723137</v>
+        <v>116.723137</v>
       </c>
     </row>
     <row r="126" ht="18" customHeight="1">
@@ -22878,7 +22878,7 @@
         <v>45957.72764497685</v>
       </c>
       <c r="AW126">
-        <v>133.544306</v>
+        <v>134.544306</v>
       </c>
     </row>
     <row r="127" ht="18" customHeight="1">
@@ -23056,7 +23056,7 @@
         <v>46038.68340863426</v>
       </c>
       <c r="AW127">
-        <v>52.588542</v>
+        <v>53.588542</v>
       </c>
     </row>
     <row r="128" ht="18" customHeight="1">
@@ -23237,7 +23237,7 @@
         <v>45842.7072899537</v>
       </c>
       <c r="AW128">
-        <v>248.564664</v>
+        <v>249.564664</v>
       </c>
     </row>
     <row r="129" ht="18" customHeight="1">
@@ -23421,7 +23421,7 @@
         <v>45868.56623082176</v>
       </c>
       <c r="AW129">
-        <v>222.705718</v>
+        <v>223.705718</v>
       </c>
     </row>
     <row r="130" ht="18" customHeight="1">
@@ -23599,7 +23599,7 @@
         <v>45890.69579123842</v>
       </c>
       <c r="AW130">
-        <v>200.576157</v>
+        <v>201.576157</v>
       </c>
     </row>
     <row r="131" ht="18" customHeight="1">
@@ -23712,7 +23712,7 @@
         <v>46079.66128135417</v>
       </c>
       <c r="AN131">
-        <v>11.610671</v>
+        <v>12.610671</v>
       </c>
     </row>
     <row r="132" ht="18" customHeight="1">
@@ -23893,7 +23893,7 @@
         <v>46086.6752787037</v>
       </c>
       <c r="AW132">
-        <v>4.596667</v>
+        <v>5.596667</v>
       </c>
     </row>
     <row r="133" ht="18" customHeight="1">
@@ -24074,7 +24074,7 @@
         <v>45904.38667092593</v>
       </c>
       <c r="AW133">
-        <v>186.885278</v>
+        <v>187.885278</v>
       </c>
     </row>
     <row r="134" ht="18" customHeight="1">
@@ -24187,7 +24187,7 @@
         <v>46056.35300378472</v>
       </c>
       <c r="AN134">
-        <v>34.918947</v>
+        <v>35.918947</v>
       </c>
     </row>
     <row r="135" ht="18" customHeight="1">
@@ -24365,7 +24365,7 @@
         <v>45826.76858534722</v>
       </c>
       <c r="AW135">
-        <v>264.503368</v>
+        <v>265.503368</v>
       </c>
     </row>
     <row r="136" ht="18" customHeight="1">
@@ -24546,7 +24546,7 @@
         <v>45986.57620032407</v>
       </c>
       <c r="AW136">
-        <v>104.695752</v>
+        <v>105.695752</v>
       </c>
     </row>
     <row r="137" ht="18" customHeight="1">
@@ -24727,7 +24727,7 @@
         <v>46002.7290687963</v>
       </c>
       <c r="AW137">
-        <v>88.54288200000001</v>
+        <v>89.54288200000001</v>
       </c>
     </row>
     <row r="138" ht="18" customHeight="1">
@@ -24900,7 +24900,7 @@
         <v>45831.67398204861</v>
       </c>
       <c r="AW138">
-        <v>259.597963</v>
+        <v>260.597963</v>
       </c>
     </row>
     <row r="139" ht="18" customHeight="1">
@@ -25081,7 +25081,7 @@
         <v>46001.47355491898</v>
       </c>
       <c r="AW139">
-        <v>89.798391</v>
+        <v>90.798391</v>
       </c>
     </row>
     <row r="140" ht="18" customHeight="1">
@@ -25262,7 +25262,7 @@
         <v>46072.59686878472</v>
       </c>
       <c r="AW140">
-        <v>18.675081</v>
+        <v>19.675081</v>
       </c>
     </row>
     <row r="141" ht="18" customHeight="1">
@@ -25443,7 +25443,7 @@
         <v>45917.46641751158</v>
       </c>
       <c r="AW141">
-        <v>173.805532</v>
+        <v>174.805532</v>
       </c>
     </row>
     <row r="142" ht="18" customHeight="1">
@@ -25624,7 +25624,7 @@
         <v>45923.31500230324</v>
       </c>
       <c r="AW142">
-        <v>167.956944</v>
+        <v>168.956944</v>
       </c>
     </row>
     <row r="143" ht="18" customHeight="1">
@@ -25802,7 +25802,7 @@
         <v>45812.58332680556</v>
       </c>
       <c r="AW143">
-        <v>277.647986</v>
+        <v>278.647986</v>
       </c>
     </row>
     <row r="144" ht="18" customHeight="1">
@@ -25980,7 +25980,7 @@
         <v>45887.78360177083</v>
       </c>
       <c r="AW144">
-        <v>203.488345</v>
+        <v>204.488345</v>
       </c>
     </row>
     <row r="145" ht="18" customHeight="1">
@@ -26161,7 +26161,7 @@
         <v>45929.32963659722</v>
       </c>
       <c r="AW145">
-        <v>161.942315</v>
+        <v>162.942315</v>
       </c>
     </row>
     <row r="146" ht="18" customHeight="1">
@@ -26337,7 +26337,7 @@
         <v>45993.4571319213</v>
       </c>
       <c r="AW146">
-        <v>97.814815</v>
+        <v>98.814815</v>
       </c>
     </row>
     <row r="147" ht="18" customHeight="1">
@@ -26518,7 +26518,7 @@
         <v>46059.43619244212</v>
       </c>
       <c r="AW147">
-        <v>31.835752</v>
+        <v>32.835752</v>
       </c>
     </row>
     <row r="148" ht="18" customHeight="1">
@@ -26696,7 +26696,7 @@
         <v>45831.62328704861</v>
       </c>
       <c r="AW148">
-        <v>259.648657</v>
+        <v>260.648657</v>
       </c>
     </row>
     <row r="149" ht="18" customHeight="1">
@@ -26874,7 +26874,7 @@
         <v>45826.76692778935</v>
       </c>
       <c r="AW149">
-        <v>264.505023</v>
+        <v>265.505023</v>
       </c>
     </row>
     <row r="150" ht="18" customHeight="1">
@@ -27008,7 +27008,7 @@
         <v>46090.5815483912</v>
       </c>
       <c r="AQ150">
-        <v>0.690405</v>
+        <v>1.690405</v>
       </c>
     </row>
     <row r="151" ht="18" customHeight="1">
@@ -27189,7 +27189,7 @@
         <v>45890.58630611112</v>
       </c>
       <c r="AW151">
-        <v>200.685648</v>
+        <v>201.685648</v>
       </c>
     </row>
     <row r="152" ht="18" customHeight="1">
@@ -27367,7 +27367,7 @@
         <v>45856.44962944444</v>
       </c>
       <c r="AW152">
-        <v>234.822326</v>
+        <v>235.822326</v>
       </c>
     </row>
     <row r="153" ht="18" customHeight="1">
@@ -27545,7 +27545,7 @@
         <v>45859.70515091435</v>
       </c>
       <c r="AW153">
-        <v>231.566794</v>
+        <v>232.566794</v>
       </c>
     </row>
     <row r="154" ht="18" customHeight="1">
@@ -27726,7 +27726,7 @@
         <v>45896.58530709491</v>
       </c>
       <c r="AW154">
-        <v>194.686644</v>
+        <v>195.686644</v>
       </c>
     </row>
     <row r="155" ht="18" customHeight="1">
@@ -27907,7 +27907,7 @@
         <v>46037.6671268287</v>
       </c>
       <c r="AW155">
-        <v>53.604826</v>
+        <v>54.604826</v>
       </c>
     </row>
     <row r="156" ht="18" customHeight="1">
@@ -28088,7 +28088,7 @@
         <v>45924.45313572917</v>
       </c>
       <c r="AW156">
-        <v>166.818819</v>
+        <v>167.818819</v>
       </c>
     </row>
     <row r="157" ht="18" customHeight="1">
@@ -28269,7 +28269,7 @@
         <v>45924.65307170139</v>
       </c>
       <c r="AW157">
-        <v>166.618877</v>
+        <v>167.618877</v>
       </c>
     </row>
     <row r="158" ht="18" customHeight="1">
@@ -28447,7 +28447,7 @@
         <v>46057.32008791667</v>
       </c>
       <c r="AW158">
-        <v>33.951863</v>
+        <v>34.951863</v>
       </c>
     </row>
     <row r="159" ht="18" customHeight="1">
@@ -28631,7 +28631,7 @@
         <v>46001.4660153125</v>
       </c>
       <c r="AW159">
-        <v>89.805938</v>
+        <v>90.805938</v>
       </c>
     </row>
     <row r="160" ht="18" customHeight="1">
@@ -28812,7 +28812,7 @@
         <v>45905.60530078704</v>
       </c>
       <c r="AW160">
-        <v>188.517014</v>
+        <v>189.517014</v>
       </c>
     </row>
     <row r="161" ht="18" customHeight="1">
@@ -29001,7 +29001,7 @@
         <v>45912.68970434028</v>
       </c>
       <c r="AW161">
-        <v>178.582245</v>
+        <v>179.582245</v>
       </c>
     </row>
     <row r="162" ht="18" customHeight="1">
@@ -29169,7 +29169,7 @@
         <v>45882.61953023148</v>
       </c>
       <c r="AW162">
-        <v>208.652419</v>
+        <v>209.652419</v>
       </c>
     </row>
     <row r="163" ht="18" customHeight="1">
@@ -29350,7 +29350,7 @@
         <v>45929.33033346065</v>
       </c>
       <c r="AW163">
-        <v>161.94162</v>
+        <v>162.94162</v>
       </c>
     </row>
     <row r="164" ht="18" customHeight="1">
@@ -29531,7 +29531,7 @@
         <v>45985.75649112268</v>
       </c>
       <c r="AW164">
-        <v>105.515463</v>
+        <v>106.515463</v>
       </c>
     </row>
     <row r="165" ht="18" customHeight="1">
@@ -29712,7 +29712,7 @@
         <v>46044.64347104167</v>
       </c>
       <c r="AW165">
-        <v>46.628484</v>
+        <v>47.628484</v>
       </c>
     </row>
     <row r="166" ht="18" customHeight="1">
@@ -29893,7 +29893,7 @@
         <v>45860.39774737268</v>
       </c>
       <c r="AW166">
-        <v>230.874201</v>
+        <v>231.874201</v>
       </c>
     </row>
     <row r="167" ht="18" customHeight="1">
@@ -30074,7 +30074,7 @@
         <v>45904.38106203704</v>
       </c>
       <c r="AW167">
-        <v>186.890891</v>
+        <v>187.890891</v>
       </c>
     </row>
     <row r="168" ht="18" customHeight="1">
@@ -30255,7 +30255,7 @@
         <v>45980.73353560185</v>
       </c>
       <c r="AW168">
-        <v>110.538414</v>
+        <v>111.538414</v>
       </c>
     </row>
     <row r="169" ht="18" customHeight="1">
@@ -30433,7 +30433,7 @@
         <v>46057.31564032407</v>
       </c>
       <c r="AW169">
-        <v>33.956308</v>
+        <v>34.956308</v>
       </c>
     </row>
     <row r="170" ht="18" customHeight="1">
@@ -30611,7 +30611,7 @@
         <v>45870.37493769676</v>
       </c>
       <c r="AW170">
-        <v>220.897014</v>
+        <v>221.897014</v>
       </c>
     </row>
     <row r="171" ht="18" customHeight="1">
@@ -30792,7 +30792,7 @@
         <v>45954.62848792824</v>
       </c>
       <c r="AW171">
-        <v>136.643461</v>
+        <v>137.643461</v>
       </c>
     </row>
     <row r="172" ht="18" customHeight="1">
@@ -30970,7 +30970,7 @@
         <v>45986.57927599538</v>
       </c>
       <c r="AW172">
-        <v>104.692674</v>
+        <v>105.692674</v>
       </c>
     </row>
     <row r="173" ht="18" customHeight="1">
@@ -31151,7 +31151,7 @@
         <v>46086.67425099537</v>
       </c>
       <c r="AW173">
-        <v>4.597697</v>
+        <v>5.597697</v>
       </c>
     </row>
     <row r="174" ht="18" customHeight="1">
@@ -31329,7 +31329,7 @@
         <v>45821.67315659721</v>
       </c>
       <c r="AW174">
-        <v>269.598796</v>
+        <v>270.598796</v>
       </c>
     </row>
     <row r="175" ht="18" customHeight="1">
@@ -31510,7 +31510,7 @@
         <v>45845.32285525464</v>
       </c>
       <c r="AW175">
-        <v>245.949097</v>
+        <v>246.949097</v>
       </c>
     </row>
     <row r="176" ht="18" customHeight="1">
@@ -31688,7 +31688,7 @@
         <v>46036.59229349537</v>
       </c>
       <c r="AW176">
-        <v>54.679653</v>
+        <v>55.679653</v>
       </c>
     </row>
     <row r="177" ht="18" customHeight="1">
@@ -31866,7 +31866,7 @@
         <v>46063.54699333334</v>
       </c>
       <c r="AW177">
-        <v>27.724954</v>
+        <v>28.724954</v>
       </c>
     </row>
     <row r="178" ht="18" customHeight="1">
@@ -32039,7 +32039,7 @@
         <v>45905.68003464121</v>
       </c>
       <c r="AW178">
-        <v>185.591921</v>
+        <v>186.591921</v>
       </c>
     </row>
     <row r="179" ht="18" customHeight="1">
@@ -32220,7 +32220,7 @@
         <v>46027.33587091435</v>
       </c>
       <c r="AW179">
-        <v>63.936076</v>
+        <v>64.936076</v>
       </c>
     </row>
     <row r="180" ht="18" customHeight="1">
@@ -32398,7 +32398,7 @@
         <v>46077.70038504629</v>
       </c>
       <c r="AW180">
-        <v>13.571563</v>
+        <v>14.571563</v>
       </c>
     </row>
     <row r="181" ht="18" customHeight="1">
@@ -32576,7 +32576,7 @@
         <v>45870.3699896875</v>
       </c>
       <c r="AW181">
-        <v>220.901956</v>
+        <v>221.901956</v>
       </c>
     </row>
     <row r="182" ht="18" customHeight="1">
@@ -32754,7 +32754,7 @@
         <v>45817.43698824074</v>
       </c>
       <c r="AW182">
-        <v>273.834965</v>
+        <v>274.834965</v>
       </c>
     </row>
     <row r="183" ht="18" customHeight="1">
@@ -32932,7 +32932,7 @@
         <v>45895.66891309028</v>
       </c>
       <c r="AW183">
-        <v>195.603032</v>
+        <v>196.603032</v>
       </c>
     </row>
     <row r="184" ht="18" customHeight="1">
@@ -33110,7 +33110,7 @@
         <v>45824.67360026621</v>
       </c>
       <c r="AW184">
-        <v>266.598345</v>
+        <v>267.598345</v>
       </c>
     </row>
     <row r="185" ht="18" customHeight="1">
@@ -33288,7 +33288,7 @@
         <v>45833.56676576388</v>
       </c>
       <c r="AW185">
-        <v>257.705185</v>
+        <v>258.705185</v>
       </c>
     </row>
     <row r="186" ht="18" customHeight="1">
@@ -33466,7 +33466,7 @@
         <v>45895.64817069445</v>
       </c>
       <c r="AW186">
-        <v>195.623785</v>
+        <v>196.623785</v>
       </c>
     </row>
     <row r="187" ht="18" customHeight="1">
@@ -33647,7 +33647,7 @@
         <v>45966.55113974537</v>
       </c>
       <c r="AW187">
-        <v>124.72081</v>
+        <v>125.72081</v>
       </c>
     </row>
     <row r="188" ht="18" customHeight="1">
@@ -33789,7 +33789,7 @@
         <v>46076.53159934028</v>
       </c>
       <c r="AQ188">
-        <v>14.740347</v>
+        <v>15.740347</v>
       </c>
     </row>
     <row r="189" ht="18" customHeight="1">
@@ -33967,7 +33967,7 @@
         <v>45824.67396405093</v>
       </c>
       <c r="AW189">
-        <v>266.597986</v>
+        <v>267.597986</v>
       </c>
     </row>
     <row r="190" ht="18" customHeight="1">
@@ -34148,7 +34148,7 @@
         <v>45868.57042331019</v>
       </c>
       <c r="AW190">
-        <v>222.701528</v>
+        <v>223.701528</v>
       </c>
     </row>
     <row r="191" ht="18" customHeight="1">
@@ -34329,7 +34329,7 @@
         <v>45923.31572024305</v>
       </c>
       <c r="AW191">
-        <v>167.956227</v>
+        <v>168.956227</v>
       </c>
     </row>
     <row r="192" ht="18" customHeight="1">
@@ -34510,7 +34510,7 @@
         <v>45890.75601248843</v>
       </c>
       <c r="AW192">
-        <v>200.515938</v>
+        <v>201.515938</v>
       </c>
     </row>
     <row r="193" ht="18" customHeight="1">
@@ -34691,7 +34691,7 @@
         <v>45979.60267356482</v>
       </c>
       <c r="AW193">
-        <v>111.669282</v>
+        <v>112.669282</v>
       </c>
     </row>
     <row r="194" ht="18" customHeight="1">
@@ -34869,7 +34869,7 @@
         <v>46057.31766871527</v>
       </c>
       <c r="AW194">
-        <v>33.954282</v>
+        <v>34.954282</v>
       </c>
     </row>
     <row r="195" ht="18" customHeight="1">
@@ -35047,7 +35047,7 @@
         <v>45817.4294139699</v>
       </c>
       <c r="AW195">
-        <v>273.842535</v>
+        <v>274.842535</v>
       </c>
     </row>
     <row r="196" ht="18" customHeight="1">
@@ -35215,7 +35215,7 @@
         <v>45882.60734775463</v>
       </c>
       <c r="AW196">
-        <v>208.664606</v>
+        <v>209.664606</v>
       </c>
     </row>
     <row r="197" ht="18" customHeight="1">
@@ -35396,7 +35396,7 @@
         <v>45904.38355210648</v>
       </c>
       <c r="AW197">
-        <v>186.888403</v>
+        <v>187.888403</v>
       </c>
     </row>
     <row r="198" ht="18" customHeight="1">
@@ -35580,7 +35580,7 @@
         <v>45905.68527717593</v>
       </c>
       <c r="AW198">
-        <v>167.959769</v>
+        <v>168.959769</v>
       </c>
     </row>
     <row r="199" ht="18" customHeight="1">
@@ -35764,7 +35764,7 @@
         <v>45868.56660532407</v>
       </c>
       <c r="AW199">
-        <v>222.705347</v>
+        <v>223.705347</v>
       </c>
     </row>
     <row r="200" ht="18" customHeight="1">
@@ -35945,7 +35945,7 @@
         <v>46001.47424234953</v>
       </c>
       <c r="AW200">
-        <v>89.797708</v>
+        <v>90.797708</v>
       </c>
     </row>
     <row r="201" ht="18" customHeight="1">
@@ -36123,7 +36123,7 @@
         <v>45824.58295356482</v>
       </c>
       <c r="AW201">
-        <v>266.688993</v>
+        <v>267.688993</v>
       </c>
     </row>
     <row r="202" ht="18" customHeight="1">
@@ -36301,7 +36301,7 @@
         <v>45810.36211870371</v>
       </c>
       <c r="AW202">
-        <v>280.909826</v>
+        <v>281.909826</v>
       </c>
     </row>
     <row r="203" ht="18" customHeight="1">
@@ -36482,7 +36482,7 @@
         <v>45904.37770018518</v>
       </c>
       <c r="AW203">
-        <v>186.894248</v>
+        <v>187.894248</v>
       </c>
     </row>
     <row r="204" ht="18" customHeight="1">
@@ -36660,7 +36660,7 @@
         <v>45930.59030788194</v>
       </c>
       <c r="AW204">
-        <v>160.681644</v>
+        <v>161.681644</v>
       </c>
     </row>
     <row r="205" ht="18" customHeight="1">
@@ -36841,7 +36841,7 @@
         <v>45810.35108107638</v>
       </c>
       <c r="AW205">
-        <v>253.925532</v>
+        <v>254.925532</v>
       </c>
     </row>
     <row r="206" ht="18" customHeight="1">
@@ -37019,7 +37019,7 @@
         <v>45826.76801165509</v>
       </c>
       <c r="AW206">
-        <v>264.503935</v>
+        <v>265.503935</v>
       </c>
     </row>
     <row r="207" ht="18" customHeight="1">
@@ -37197,7 +37197,7 @@
         <v>45898.66446734954</v>
       </c>
       <c r="AW207">
-        <v>192.607488</v>
+        <v>193.607488</v>
       </c>
     </row>
     <row r="208" ht="18" customHeight="1">
@@ -37375,7 +37375,7 @@
         <v>46073.66776079861</v>
       </c>
       <c r="AW208">
-        <v>17.60419</v>
+        <v>18.60419</v>
       </c>
     </row>
     <row r="209" ht="18" customHeight="1">
@@ -37556,7 +37556,7 @@
         <v>45842.71044888889</v>
       </c>
       <c r="AW209">
-        <v>248.561505</v>
+        <v>249.561505</v>
       </c>
     </row>
     <row r="210" ht="18" customHeight="1">
@@ -37737,7 +37737,7 @@
         <v>45880.49447488426</v>
       </c>
       <c r="AW210">
-        <v>196.530926</v>
+        <v>197.530926</v>
       </c>
     </row>
     <row r="211" ht="18" customHeight="1">
@@ -37915,7 +37915,7 @@
         <v>46036.58667920139</v>
       </c>
       <c r="AW211">
-        <v>54.685266</v>
+        <v>55.685266</v>
       </c>
     </row>
     <row r="212" ht="18" customHeight="1">
@@ -38093,7 +38093,7 @@
         <v>45821.69981792824</v>
       </c>
       <c r="AW212">
-        <v>269.57213</v>
+        <v>270.57213</v>
       </c>
     </row>
     <row r="213" ht="18" customHeight="1">
@@ -38206,7 +38206,7 @@
         <v>46079.66134925926</v>
       </c>
       <c r="AN213">
-        <v>11.610602</v>
+        <v>12.610602</v>
       </c>
     </row>
     <row r="214" ht="18" customHeight="1">
@@ -38384,7 +38384,7 @@
         <v>45824.58350305556</v>
       </c>
       <c r="AW214">
-        <v>266.688449</v>
+        <v>267.688449</v>
       </c>
     </row>
     <row r="215" ht="18" customHeight="1">
@@ -38562,7 +38562,7 @@
         <v>46090.73012363426</v>
       </c>
       <c r="AW215">
-        <v>0.541829</v>
+        <v>1.541829</v>
       </c>
     </row>
     <row r="216" ht="18" customHeight="1">
@@ -38740,7 +38740,7 @@
         <v>45825.66128076389</v>
       </c>
       <c r="AW216">
-        <v>265.610671</v>
+        <v>266.610671</v>
       </c>
     </row>
     <row r="217" ht="18" customHeight="1">
@@ -38918,7 +38918,7 @@
         <v>45813.67869909722</v>
       </c>
       <c r="AW217">
-        <v>277.593252</v>
+        <v>278.593252</v>
       </c>
     </row>
     <row r="218" ht="18" customHeight="1">
@@ -39096,7 +39096,7 @@
         <v>45811.53830461806</v>
       </c>
       <c r="AW218">
-        <v>279.733646</v>
+        <v>280.733646</v>
       </c>
     </row>
     <row r="219" ht="18" customHeight="1">
@@ -39274,7 +39274,7 @@
         <v>45821.62512202546</v>
       </c>
       <c r="AW219">
-        <v>269.646829</v>
+        <v>270.646829</v>
       </c>
     </row>
     <row r="220" ht="18" customHeight="1">
@@ -39452,7 +39452,7 @@
         <v>45859.70342961806</v>
       </c>
       <c r="AW220">
-        <v>231.568519</v>
+        <v>232.568519</v>
       </c>
     </row>
     <row r="221" ht="18" customHeight="1">
@@ -39633,7 +39633,7 @@
         <v>45859.68545269676</v>
       </c>
       <c r="AW221">
-        <v>231.586493</v>
+        <v>232.586493</v>
       </c>
     </row>
     <row r="222" ht="18" customHeight="1">
@@ -39814,7 +39814,7 @@
         <v>45954.36042099537</v>
       </c>
       <c r="AW222">
-        <v>136.911528</v>
+        <v>137.911528</v>
       </c>
     </row>
     <row r="223" ht="18" customHeight="1">
@@ -39956,7 +39956,7 @@
         <v>46076.53141864583</v>
       </c>
       <c r="AQ223">
-        <v>14.740532</v>
+        <v>15.740532</v>
       </c>
     </row>
     <row r="224" ht="18" customHeight="1">
@@ -40134,7 +40134,7 @@
         <v>45812.58297493056</v>
       </c>
       <c r="AW224">
-        <v>278.68897</v>
+        <v>279.68897</v>
       </c>
     </row>
     <row r="225" ht="18" customHeight="1">
@@ -40312,7 +40312,7 @@
         <v>45821.68405166667</v>
       </c>
       <c r="AW225">
-        <v>269.587894</v>
+        <v>270.587894</v>
       </c>
     </row>
     <row r="226" ht="18" customHeight="1">
@@ -40490,7 +40490,7 @@
         <v>45812.58710694444</v>
       </c>
       <c r="AW226">
-        <v>278.684838</v>
+        <v>279.684838</v>
       </c>
     </row>
     <row r="227" ht="18" customHeight="1">
@@ -40671,7 +40671,7 @@
         <v>45911.63280706019</v>
       </c>
       <c r="AW227">
-        <v>179.639144</v>
+        <v>180.639144</v>
       </c>
     </row>
     <row r="228" ht="18" customHeight="1">
@@ -40852,7 +40852,7 @@
         <v>45979.57851665509</v>
       </c>
       <c r="AW228">
-        <v>111.693438</v>
+        <v>112.693438</v>
       </c>
     </row>
     <row r="229" ht="18" customHeight="1">
@@ -41033,7 +41033,7 @@
         <v>45986.56036744213</v>
       </c>
       <c r="AW229">
-        <v>104.711586</v>
+        <v>105.711586</v>
       </c>
     </row>
     <row r="230" ht="18" customHeight="1">
@@ -41214,7 +41214,7 @@
         <v>46051.33887575231</v>
       </c>
       <c r="AW230">
-        <v>39.933079</v>
+        <v>40.933079</v>
       </c>
     </row>
     <row r="231" ht="18" customHeight="1">
@@ -41395,7 +41395,7 @@
         <v>46051.33719802083</v>
       </c>
       <c r="AW231">
-        <v>39.934757</v>
+        <v>40.934757</v>
       </c>
     </row>
     <row r="232" ht="18" customHeight="1">
@@ -41576,7 +41576,7 @@
         <v>45904.37834540509</v>
       </c>
       <c r="AW232">
-        <v>186.8936</v>
+        <v>187.8936</v>
       </c>
     </row>
     <row r="233" ht="18" customHeight="1">
@@ -41757,7 +41757,7 @@
         <v>45820.33415019676</v>
       </c>
       <c r="AW233">
-        <v>238.659074</v>
+        <v>239.659074</v>
       </c>
     </row>
     <row r="234" ht="18" customHeight="1">
@@ -41935,7 +41935,7 @@
         <v>45835.37156861111</v>
       </c>
       <c r="AW234">
-        <v>255.900382</v>
+        <v>256.900382</v>
       </c>
     </row>
     <row r="235" ht="18" customHeight="1">
@@ -42116,7 +42116,7 @@
         <v>45895.60195914352</v>
       </c>
       <c r="AW235">
-        <v>195.669988</v>
+        <v>196.669988</v>
       </c>
     </row>
     <row r="236" ht="18" customHeight="1">
@@ -42300,7 +42300,7 @@
         <v>45903.36175993056</v>
       </c>
       <c r="AW236">
-        <v>187.910185</v>
+        <v>188.910185</v>
       </c>
     </row>
     <row r="237" ht="18" customHeight="1">
@@ -42481,7 +42481,7 @@
         <v>45923.31386627315</v>
       </c>
       <c r="AW237">
-        <v>167.958079</v>
+        <v>168.958079</v>
       </c>
     </row>
     <row r="238" ht="18" customHeight="1">
@@ -42659,7 +42659,7 @@
         <v>45972.38501128473</v>
       </c>
       <c r="AW238">
-        <v>118.886944</v>
+        <v>119.886944</v>
       </c>
     </row>
     <row r="239" ht="18" customHeight="1">
@@ -42840,7 +42840,7 @@
         <v>46086.67639361111</v>
       </c>
       <c r="AW239">
-        <v>4.595556</v>
+        <v>5.595556</v>
       </c>
     </row>
     <row r="240" ht="18" customHeight="1">
@@ -43021,7 +43021,7 @@
         <v>45860.39721776621</v>
       </c>
       <c r="AW240">
-        <v>230.874734</v>
+        <v>231.874734</v>
       </c>
     </row>
     <row r="241" ht="18" customHeight="1">
@@ -43202,7 +43202,7 @@
         <v>45904.51875018519</v>
       </c>
       <c r="AW241">
-        <v>186.753194</v>
+        <v>187.753194</v>
       </c>
     </row>
     <row r="242" ht="18" customHeight="1">
@@ -43383,7 +43383,7 @@
         <v>46001.47301980324</v>
       </c>
       <c r="AW242">
-        <v>89.798935</v>
+        <v>90.798935</v>
       </c>
     </row>
     <row r="243" ht="18" customHeight="1">
@@ -43561,7 +43561,7 @@
         <v>46036.59334578704</v>
       </c>
       <c r="AW243">
-        <v>54.6786</v>
+        <v>55.6786</v>
       </c>
     </row>
     <row r="244" ht="18" customHeight="1">
@@ -43742,7 +43742,7 @@
         <v>45985.7559840162</v>
       </c>
       <c r="AW244">
-        <v>105.515961</v>
+        <v>106.515961</v>
       </c>
     </row>
     <row r="245" ht="18" customHeight="1">
@@ -43923,7 +43923,7 @@
         <v>45820.33046670139</v>
       </c>
       <c r="AW245">
-        <v>220.900729</v>
+        <v>221.900729</v>
       </c>
     </row>
     <row r="246" ht="18" customHeight="1">
@@ -44096,7 +44096,7 @@
         <v>45824.69872459491</v>
       </c>
       <c r="AW246">
-        <v>266.573229</v>
+        <v>267.573229</v>
       </c>
     </row>
     <row r="247" ht="18" customHeight="1">
@@ -44274,7 +44274,7 @@
         <v>45859.70464324074</v>
       </c>
       <c r="AW247">
-        <v>231.567303</v>
+        <v>232.567303</v>
       </c>
     </row>
     <row r="248" ht="18" customHeight="1">
@@ -44458,7 +44458,7 @@
         <v>45895.67057834491</v>
       </c>
       <c r="AW248">
-        <v>195.601377</v>
+        <v>196.601377</v>
       </c>
     </row>
     <row r="249" ht="18" customHeight="1">
@@ -44639,7 +44639,7 @@
         <v>45952.41598819445</v>
       </c>
       <c r="AW249">
-        <v>138.855961</v>
+        <v>139.855961</v>
       </c>
     </row>
     <row r="250" ht="18" customHeight="1">
@@ -44823,7 +44823,7 @@
         <v>45923.57573010417</v>
       </c>
       <c r="AW250">
-        <v>167.660845</v>
+        <v>168.660845</v>
       </c>
     </row>
     <row r="251" ht="18" customHeight="1">
@@ -45004,7 +45004,7 @@
         <v>45929.33121140047</v>
       </c>
       <c r="AW251">
-        <v>161.940741</v>
+        <v>162.940741</v>
       </c>
     </row>
     <row r="252" ht="18" customHeight="1">
@@ -45185,7 +45185,7 @@
         <v>46078.55240465277</v>
       </c>
       <c r="AW252">
-        <v>12.719549</v>
+        <v>13.719549</v>
       </c>
     </row>
     <row r="253" ht="18" customHeight="1">
@@ -45363,7 +45363,7 @@
         <v>45859.70424362268</v>
       </c>
       <c r="AW253">
-        <v>231.567708</v>
+        <v>232.567708</v>
       </c>
     </row>
     <row r="254" ht="18" customHeight="1">
@@ -45544,7 +45544,7 @@
         <v>45888.4437121875</v>
       </c>
       <c r="AW254">
-        <v>202.828241</v>
+        <v>203.828241</v>
       </c>
     </row>
     <row r="255" ht="18" customHeight="1">
@@ -45725,7 +45725,7 @@
         <v>46051.59352782407</v>
       </c>
       <c r="AW255">
-        <v>39.678426</v>
+        <v>40.678426</v>
       </c>
     </row>
     <row r="256" ht="18" customHeight="1">
@@ -45906,7 +45906,7 @@
         <v>45839.55104972223</v>
       </c>
       <c r="AW256">
-        <v>251.720903</v>
+        <v>252.720903</v>
       </c>
     </row>
     <row r="257" ht="18" customHeight="1">
@@ -46087,7 +46087,7 @@
         <v>46050.54756696759</v>
       </c>
       <c r="AW257">
-        <v>40.724387</v>
+        <v>41.724387</v>
       </c>
     </row>
     <row r="258" ht="18" customHeight="1">
@@ -46188,7 +46188,7 @@
         <v>46076.60415833333</v>
       </c>
       <c r="AK258">
-        <v>14.667789</v>
+        <v>15.667789</v>
       </c>
     </row>
     <row r="259" ht="18" customHeight="1">
@@ -46289,7 +46289,7 @@
         <v>46076.70991956018</v>
       </c>
       <c r="AK259">
-        <v>14.562025</v>
+        <v>15.562025</v>
       </c>
     </row>
     <row r="260" ht="18" customHeight="1">
@@ -46470,7 +46470,7 @@
         <v>46027.33658649305</v>
       </c>
       <c r="AW260">
-        <v>63.935359</v>
+        <v>64.93535900000001</v>
       </c>
     </row>
     <row r="261" ht="18" customHeight="1">
@@ -46651,7 +46651,7 @@
         <v>45860.43664048611</v>
       </c>
       <c r="AW261">
-        <v>230.835313</v>
+        <v>231.835313</v>
       </c>
     </row>
     <row r="262" ht="18" customHeight="1">
@@ -46829,7 +46829,7 @@
         <v>45929.32146375</v>
       </c>
       <c r="AW262">
-        <v>161.950486</v>
+        <v>162.950486</v>
       </c>
     </row>
     <row r="263" ht="18" customHeight="1">
@@ -47010,7 +47010,7 @@
         <v>45929.3236115625</v>
       </c>
       <c r="AW263">
-        <v>161.948333</v>
+        <v>162.948333</v>
       </c>
     </row>
     <row r="264" ht="18" customHeight="1">
@@ -47188,7 +47188,7 @@
         <v>45954.73906835648</v>
       </c>
       <c r="AW264">
-        <v>136.532882</v>
+        <v>137.532882</v>
       </c>
     </row>
     <row r="265" ht="18" customHeight="1">
@@ -47364,7 +47364,7 @@
         <v>45862.4923733912</v>
       </c>
       <c r="AW265">
-        <v>228.779572</v>
+        <v>229.779572</v>
       </c>
     </row>
     <row r="266" ht="18" customHeight="1">
@@ -47542,7 +47542,7 @@
         <v>45938.33289437499</v>
       </c>
       <c r="AW266">
-        <v>152.939051</v>
+        <v>153.939051</v>
       </c>
     </row>
     <row r="267" ht="18" customHeight="1">
@@ -47726,7 +47726,7 @@
         <v>45946.65466756944</v>
       </c>
       <c r="AW267">
-        <v>138.711273</v>
+        <v>139.711273</v>
       </c>
     </row>
     <row r="268" ht="18" customHeight="1">
@@ -47904,7 +47904,7 @@
         <v>46003.56398351852</v>
       </c>
       <c r="AW268">
-        <v>87.70796300000001</v>
+        <v>88.70796300000001</v>
       </c>
     </row>
     <row r="269" ht="18" customHeight="1">
@@ -48085,7 +48085,7 @@
         <v>45831.5739419676</v>
       </c>
       <c r="AW269">
-        <v>259.698009</v>
+        <v>260.698009</v>
       </c>
     </row>
     <row r="270" ht="18" customHeight="1">
@@ -48263,7 +48263,7 @@
         <v>45821.62585732639</v>
       </c>
       <c r="AW270">
-        <v>269.646088</v>
+        <v>270.646088</v>
       </c>
     </row>
     <row r="271" ht="18" customHeight="1">
@@ -48444,7 +48444,7 @@
         <v>45842.71009863426</v>
       </c>
       <c r="AW271">
-        <v>248.561852</v>
+        <v>249.561852</v>
       </c>
     </row>
     <row r="272" ht="18" customHeight="1">
@@ -48625,7 +48625,7 @@
         <v>45966.55123927083</v>
       </c>
       <c r="AW272">
-        <v>124.720706</v>
+        <v>125.720706</v>
       </c>
     </row>
     <row r="273" ht="18" customHeight="1">
@@ -48803,7 +48803,7 @@
         <v>45952.55986858797</v>
       </c>
       <c r="AW273">
-        <v>138.712083</v>
+        <v>139.712083</v>
       </c>
     </row>
     <row r="274" ht="18" customHeight="1">
@@ -48984,7 +48984,7 @@
         <v>45986.57647679398</v>
       </c>
       <c r="AW274">
-        <v>104.695475</v>
+        <v>105.695475</v>
       </c>
     </row>
     <row r="275" ht="18" customHeight="1">
@@ -49165,7 +49165,7 @@
         <v>45842.7095575463</v>
       </c>
       <c r="AW275">
-        <v>248.562396</v>
+        <v>249.562396</v>
       </c>
     </row>
     <row r="276" ht="18" customHeight="1">
@@ -49343,7 +49343,7 @@
         <v>45923.31946878473</v>
       </c>
       <c r="AW276">
-        <v>167.952477</v>
+        <v>168.952477</v>
       </c>
     </row>
     <row r="277" ht="18" customHeight="1">
@@ -49527,7 +49527,7 @@
         <v>45971.57262901621</v>
       </c>
       <c r="AW277">
-        <v>119.699317</v>
+        <v>120.699317</v>
       </c>
     </row>
     <row r="278" ht="18" customHeight="1">
@@ -49708,7 +49708,7 @@
         <v>45832.68075126158</v>
       </c>
       <c r="AW278">
-        <v>258.591204</v>
+        <v>259.591204</v>
       </c>
     </row>
     <row r="279" ht="18" customHeight="1">
@@ -49889,7 +49889,7 @@
         <v>45917.46522068288</v>
       </c>
       <c r="AW279">
-        <v>173.806725</v>
+        <v>174.806725</v>
       </c>
     </row>
     <row r="280" ht="18" customHeight="1">
@@ -50070,7 +50070,7 @@
         <v>45986.55970949074</v>
       </c>
       <c r="AW280">
-        <v>104.712245</v>
+        <v>105.712245</v>
       </c>
     </row>
     <row r="281" ht="18" customHeight="1">
@@ -50251,7 +50251,7 @@
         <v>45965.37861903935</v>
       </c>
       <c r="AW281">
-        <v>125.893333</v>
+        <v>126.893333</v>
       </c>
     </row>
     <row r="282" ht="18" customHeight="1">
@@ -50432,7 +50432,7 @@
         <v>45846.4887596412</v>
       </c>
       <c r="AW282">
-        <v>244.783194</v>
+        <v>245.783194</v>
       </c>
     </row>
     <row r="283" ht="18" customHeight="1">
@@ -50639,7 +50639,7 @@
         <v>45966.44556553241</v>
       </c>
       <c r="AW283">
-        <v>124.826389</v>
+        <v>125.826389</v>
       </c>
     </row>
     <row r="284" ht="18" customHeight="1">
@@ -50817,7 +50817,7 @@
         <v>45975.64955575232</v>
       </c>
       <c r="AW284">
-        <v>115.622396</v>
+        <v>116.622396</v>
       </c>
     </row>
     <row r="285" ht="18" customHeight="1">
@@ -50998,7 +50998,7 @@
         <v>45992.61684608796</v>
       </c>
       <c r="AW285">
-        <v>98.65510399999999</v>
+        <v>99.65510399999999</v>
       </c>
     </row>
     <row r="286" ht="18" customHeight="1">
@@ -51182,7 +51182,7 @@
         <v>45924.33433900463</v>
       </c>
       <c r="AW286">
-        <v>153.942477</v>
+        <v>154.942477</v>
       </c>
     </row>
     <row r="287" ht="18" customHeight="1">
@@ -51316,7 +51316,7 @@
         <v>46090.58126142361</v>
       </c>
       <c r="AQ287">
-        <v>0.690694</v>
+        <v>1.690694</v>
       </c>
     </row>
     <row r="288" ht="18" customHeight="1">
@@ -51494,7 +51494,7 @@
         <v>45845.32248731481</v>
       </c>
       <c r="AW288">
-        <v>245.949468</v>
+        <v>246.949468</v>
       </c>
     </row>
     <row r="289" ht="18" customHeight="1">
@@ -51672,7 +51672,7 @@
         <v>45833.56582039352</v>
       </c>
       <c r="AW289">
-        <v>257.706134</v>
+        <v>258.706134</v>
       </c>
     </row>
     <row r="290" ht="18" customHeight="1">
@@ -51850,7 +51850,7 @@
         <v>45870.37016001157</v>
       </c>
       <c r="AW290">
-        <v>220.901794</v>
+        <v>221.901794</v>
       </c>
     </row>
     <row r="291" ht="18" customHeight="1">
@@ -52031,7 +52031,7 @@
         <v>45890.64208997686</v>
       </c>
       <c r="AW291">
-        <v>200.629861</v>
+        <v>201.629861</v>
       </c>
     </row>
     <row r="292" ht="18" customHeight="1">
@@ -52215,7 +52215,7 @@
         <v>45944.44625667824</v>
       </c>
       <c r="AW292">
-        <v>141.95728</v>
+        <v>142.95728</v>
       </c>
     </row>
     <row r="293" ht="18" customHeight="1">
@@ -52396,7 +52396,7 @@
         <v>45971.57897849537</v>
       </c>
       <c r="AW293">
-        <v>119.692975</v>
+        <v>120.692975</v>
       </c>
     </row>
     <row r="294" ht="18" customHeight="1">
@@ -52577,7 +52577,7 @@
         <v>45846.36008232638</v>
       </c>
       <c r="AW294">
-        <v>244.911863</v>
+        <v>245.911863</v>
       </c>
     </row>
     <row r="295" ht="18" customHeight="1">
@@ -52755,7 +52755,7 @@
         <v>45832.3608832176</v>
       </c>
       <c r="AW295">
-        <v>258.911065</v>
+        <v>259.911065</v>
       </c>
     </row>
     <row r="296" ht="18" customHeight="1">
@@ -52936,7 +52936,7 @@
         <v>45887.75298732638</v>
       </c>
       <c r="AW296">
-        <v>203.518958</v>
+        <v>204.518958</v>
       </c>
     </row>
     <row r="297" ht="18" customHeight="1">
@@ -53114,7 +53114,7 @@
         <v>45826.76998138889</v>
       </c>
       <c r="AW297">
-        <v>264.501968</v>
+        <v>265.501968</v>
       </c>
     </row>
     <row r="298" ht="18" customHeight="1">
@@ -53295,7 +53295,7 @@
         <v>45904.37713482638</v>
       </c>
       <c r="AW298">
-        <v>186.894815</v>
+        <v>187.894815</v>
       </c>
     </row>
     <row r="299" ht="18" customHeight="1">
@@ -53309,7 +53309,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Validação</t>
+          <t>Publicar na plataforma</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -53329,7 +53329,7 @@
         <v>46045.58498351852</v>
       </c>
       <c r="J299" s="2">
-        <v>46090.72899315972</v>
+        <v>46091.62691195602</v>
       </c>
       <c r="M299" s="2">
         <v>46075.58498351852</v>
@@ -53405,6 +53405,21 @@
           <t>https://docs.google.com/document/d/1ERSO1B7ZDvm0nQO6fx1fC6rTnKmNWXqnuUCTRdqjYbc/edit?tab=t.aspbfo3qvjqw</t>
         </is>
       </c>
+      <c r="AC299" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="AD299" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="AE299" t="inlineStr">
+        <is>
+          <t>Aprovado: Publicar !</t>
+        </is>
+      </c>
       <c r="AF299" t="inlineStr">
         <is>
           <t>Gestão</t>
@@ -53431,8 +53446,17 @@
       <c r="AO299" s="2">
         <v>46090.72898921296</v>
       </c>
+      <c r="AP299" s="2">
+        <v>46091.62691219908</v>
+      </c>
       <c r="AQ299">
-        <v>0.542963</v>
+        <v>0.897917</v>
+      </c>
+      <c r="AR299" s="2">
+        <v>46091.62691277778</v>
+      </c>
+      <c r="AT299">
+        <v>0.645035</v>
       </c>
     </row>
     <row r="300" ht="18" customHeight="1">
@@ -53613,7 +53637,7 @@
         <v>45986.70824453703</v>
       </c>
       <c r="AW300">
-        <v>104.563704</v>
+        <v>105.563704</v>
       </c>
     </row>
     <row r="301" ht="18" customHeight="1">
@@ -53791,7 +53815,7 @@
         <v>45859.70231407408</v>
       </c>
       <c r="AW301">
-        <v>231.569641</v>
+        <v>232.569641</v>
       </c>
     </row>
     <row r="302" ht="18" customHeight="1">
@@ -53925,7 +53949,7 @@
         <v>46090.58068733796</v>
       </c>
       <c r="AQ302">
-        <v>0.691262</v>
+        <v>1.691262</v>
       </c>
     </row>
     <row r="303" ht="18" customHeight="1">
@@ -54114,7 +54138,7 @@
         <v>45835.37110386574</v>
       </c>
       <c r="AW303">
-        <v>255.900845</v>
+        <v>256.900845</v>
       </c>
     </row>
     <row r="304" ht="18" customHeight="1">
@@ -54295,7 +54319,7 @@
         <v>45904.38426976852</v>
       </c>
       <c r="AW304">
-        <v>186.887685</v>
+        <v>187.887685</v>
       </c>
     </row>
     <row r="305" ht="18" customHeight="1">
@@ -54473,7 +54497,7 @@
         <v>45929.57279483796</v>
       </c>
       <c r="AW305">
-        <v>161.699155</v>
+        <v>162.699155</v>
       </c>
     </row>
     <row r="306" ht="18" customHeight="1">
@@ -54654,7 +54678,7 @@
         <v>46007.42707763889</v>
       </c>
       <c r="AW306">
-        <v>83.84487300000001</v>
+        <v>84.84487300000001</v>
       </c>
     </row>
     <row r="307" ht="18" customHeight="1">
@@ -54840,7 +54864,7 @@
         <v>45894.61132443287</v>
       </c>
       <c r="AW307">
-        <v>196.660625</v>
+        <v>197.660625</v>
       </c>
     </row>
     <row r="308" ht="18" customHeight="1">
@@ -55018,7 +55042,7 @@
         <v>45820.33137869213</v>
       </c>
       <c r="AW308">
-        <v>270.940567</v>
+        <v>271.940567</v>
       </c>
     </row>
     <row r="309" ht="18" customHeight="1">
@@ -55199,7 +55223,7 @@
         <v>45930.65916848379</v>
       </c>
       <c r="AW309">
-        <v>160.612778</v>
+        <v>161.612778</v>
       </c>
     </row>
     <row r="310" ht="18" customHeight="1">
@@ -55380,7 +55404,7 @@
         <v>45975.54895935186</v>
       </c>
       <c r="AW310">
-        <v>115.722986</v>
+        <v>116.722986</v>
       </c>
     </row>
     <row r="311" ht="18" customHeight="1">
@@ -55561,7 +55585,7 @@
         <v>46001.46150133102</v>
       </c>
       <c r="AW311">
-        <v>89.810451</v>
+        <v>90.810451</v>
       </c>
     </row>
     <row r="312" ht="18" customHeight="1">
@@ -55742,7 +55766,7 @@
         <v>46027.33476094907</v>
       </c>
       <c r="AW312">
-        <v>63.937188</v>
+        <v>64.93718800000001</v>
       </c>
     </row>
     <row r="313" ht="18" customHeight="1">
@@ -55923,7 +55947,7 @@
         <v>45930.6606075926</v>
       </c>
       <c r="AW313">
-        <v>160.611343</v>
+        <v>161.611343</v>
       </c>
     </row>
     <row r="314" ht="18" customHeight="1">
@@ -56104,7 +56128,7 @@
         <v>45930.65883226852</v>
       </c>
       <c r="AW314">
-        <v>160.613113</v>
+        <v>161.613113</v>
       </c>
     </row>
     <row r="315" ht="18" customHeight="1">
@@ -56205,7 +56229,7 @@
         <v>46076.70818526621</v>
       </c>
       <c r="AK315">
-        <v>14.563762</v>
+        <v>15.563762</v>
       </c>
     </row>
     <row r="316" ht="18" customHeight="1">
@@ -56383,7 +56407,7 @@
         <v>45826.76959586806</v>
       </c>
       <c r="AW316">
-        <v>264.50235</v>
+        <v>265.50235</v>
       </c>
     </row>
     <row r="317" ht="18" customHeight="1">
@@ -56561,7 +56585,7 @@
         <v>46057.31336575231</v>
       </c>
       <c r="AW317">
-        <v>33.958588</v>
+        <v>34.958588</v>
       </c>
     </row>
     <row r="318" ht="18" customHeight="1">
@@ -56742,16 +56766,16 @@
         <v>45873.70791493055</v>
       </c>
       <c r="AW318">
-        <v>217.564039</v>
+        <v>218.564039</v>
       </c>
     </row>
     <row r="319" ht="18" customHeight="1">
       <c r="A319">
-        <v>1210318748</v>
+        <v>1289597864</v>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Curso: Pós Corte Online Turma: 21 Disciplina: Princípios da gestão eficiente Tópico: Gestão economico-financeira em fazendas Professor: Guilherme Campos De Arruda LamegoData: 45980</t>
+          <t>Curso: Pós Gestão Fazendas Online Turma: 1 Disciplina: Aplicação de ferramentas e métodos de gestão Tópico: Gestão da rotina de trabalho do dia a dia, qualidade, metas e rituais de gestão Professor: Rafael Silva Alves de OliveiraTipo de Conteúdo: Onli</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -56761,11 +56785,11 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Reprovado na Validação</t>
+          <t>Gestão</t>
         </is>
       </c>
       <c r="E319" s="2">
-        <v>45979.875</v>
+        <v>46077.87559027778</v>
       </c>
       <c r="F319" t="inlineStr">
         <is>
@@ -56773,16 +56797,13 @@
         </is>
       </c>
       <c r="H319" s="2">
-        <v>45954.62754259259</v>
+        <v>46077.70090876157</v>
       </c>
       <c r="I319" s="2">
-        <v>45908.53443530093</v>
+        <v>46050.61468201389</v>
       </c>
       <c r="J319" s="2">
-        <v>45954.62754267361</v>
-      </c>
-      <c r="M319" s="2">
-        <v>45938.53443530093</v>
+        <v>46077.70090884259</v>
       </c>
       <c r="N319" t="b">
         <v>0</v>
@@ -56794,65 +56815,65 @@
       </c>
       <c r="P319" t="inlineStr">
         <is>
-          <t>Guilherme Campos De Arruda Lamego</t>
+          <t>Rafael Silva Alves de Oliveira</t>
         </is>
       </c>
       <c r="Q319" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="R319" t="inlineStr">
         <is>
-          <t>Corte</t>
+          <t>Gestão</t>
         </is>
       </c>
       <c r="S319" t="inlineStr">
         <is>
-          <t>Curso: Pós Corte Online Turma: 21 Disciplina: Princípios da gestão eficiente Tópico: Gestão economico-financeira em fazendas Professor: Guilherme Campos De Arruda LamegoData: 45980</t>
+          <t>Curso: Pós Gestão Fazendas Online Turma: 1 Disciplina: Aplicação de ferramentas e métodos de gestão Tópico: Gestão da rotina de trabalho do dia a dia, qualidade, metas e rituais de gestão Professor: Rafael Silva Alves de OliveiraTipo de Conteúdo: Onli</t>
         </is>
       </c>
       <c r="T319" t="inlineStr">
         <is>
-          <t>Pós Corte Online</t>
+          <t>Pós Gestão Fazendas Online</t>
         </is>
       </c>
       <c r="U319" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>1</t>
         </is>
       </c>
       <c r="V319" t="inlineStr">
         <is>
-          <t>Princípios da gestão eficiente</t>
+          <t>Aplicação de ferramentas e métodos de gestão</t>
         </is>
       </c>
       <c r="W319" t="inlineStr">
         <is>
-          <t>Gestão economico-financeira em fazendas</t>
+          <t>Gestão da rotina de trabalho do dia a dia, qualidade, metas e rituais de gestão</t>
         </is>
       </c>
       <c r="X319" s="2">
-        <v>45979.875</v>
+        <v>46077.87559027778</v>
       </c>
       <c r="Y319" t="inlineStr">
         <is>
-          <t>2025-10-29</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="Z319" t="inlineStr">
         <is>
-          <t>2025-11-05</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="AA319" t="inlineStr">
         <is>
-          <t>https://rehagro.instructure.com/courses/2941/modules</t>
+          <t>https://rehagro.instructure.com/courses/2974</t>
         </is>
       </c>
       <c r="AB319" t="inlineStr">
         <is>
-          <t>https://docs.google.com/document/d/1xcQZxZVIuqxticMYNr2yoDazsNBgfX4BPdfry9LsfBo/edit?tab=t.19lbzndilb0h</t>
+          <t>https://docs.google.com/document/d/1ERSO1B7ZDvm0nQO6fx1fC6rTnKmNWXqnuUCTRdqjYbc/edit?tab=t.a7jzuflcbwlc</t>
         </is>
       </c>
       <c r="AC319" t="inlineStr">
@@ -56872,67 +56893,67 @@
       </c>
       <c r="AF319" t="inlineStr">
         <is>
-          <t>Reprovado na Validação</t>
+          <t>Gestão</t>
         </is>
       </c>
       <c r="AG319" t="inlineStr">
         <is>
-          <t>01:47:00</t>
+          <t>01:49:00</t>
         </is>
       </c>
       <c r="AH319">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="AI319" s="2">
-        <v>45908.53444015046</v>
+        <v>46050.61468837963</v>
       </c>
       <c r="AJ319" s="2">
-        <v>45947.59307728009</v>
+        <v>46072.42328466436</v>
       </c>
       <c r="AK319">
-        <v>39.058634</v>
+        <v>21.808588</v>
       </c>
       <c r="AL319" s="2">
-        <v>45947.59307776621</v>
+        <v>46072.42328561343</v>
       </c>
       <c r="AM319" s="2">
-        <v>45952.56312944445</v>
+        <v>46076.34390538195</v>
       </c>
       <c r="AN319">
-        <v>1.110625</v>
+        <v>3.920613</v>
       </c>
       <c r="AO319" s="2">
-        <v>45947.59427358797</v>
+        <v>46076.34390559028</v>
       </c>
       <c r="AP319" s="2">
-        <v>45952.67415577546</v>
+        <v>46077.68847505787</v>
       </c>
       <c r="AQ319">
-        <v>3.97044</v>
+        <v>1.34456</v>
       </c>
       <c r="AR319" s="2">
-        <v>45952.67415603009</v>
+        <v>46077.68847538195</v>
       </c>
       <c r="AS319" s="2">
-        <v>45954.62754299769</v>
+        <v>46077.70090915509</v>
       </c>
       <c r="AT319">
-        <v>1.95338</v>
+        <v>0.012431</v>
       </c>
       <c r="AU319" s="2">
-        <v>45954.62754329861</v>
+        <v>46077.70090952546</v>
       </c>
       <c r="AW319">
-        <v>136.64441</v>
+        <v>14.571042</v>
       </c>
     </row>
     <row r="320" ht="18" customHeight="1">
       <c r="A320">
-        <v>1289597864</v>
+        <v>1210318748</v>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Curso: Pós Gestão Fazendas Online Turma: 1 Disciplina: Aplicação de ferramentas e métodos de gestão Tópico: Gestão da rotina de trabalho do dia a dia, qualidade, metas e rituais de gestão Professor: Rafael Silva Alves de OliveiraTipo de Conteúdo: Onli</t>
+          <t>Curso: Pós Corte Online Turma: 21 Disciplina: Princípios da gestão eficiente Tópico: Gestão economico-financeira em fazendas Professor: Guilherme Campos De Arruda LamegoData: 45980</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -56942,11 +56963,11 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Gestão</t>
+          <t>Reprovado na Validação</t>
         </is>
       </c>
       <c r="E320" s="2">
-        <v>46077.87559027778</v>
+        <v>45979.875</v>
       </c>
       <c r="F320" t="inlineStr">
         <is>
@@ -56954,13 +56975,16 @@
         </is>
       </c>
       <c r="H320" s="2">
-        <v>46077.70090876157</v>
+        <v>45954.62754259259</v>
       </c>
       <c r="I320" s="2">
-        <v>46050.61468201389</v>
+        <v>45908.53443530093</v>
       </c>
       <c r="J320" s="2">
-        <v>46077.70090884259</v>
+        <v>45954.62754267361</v>
+      </c>
+      <c r="M320" s="2">
+        <v>45938.53443530093</v>
       </c>
       <c r="N320" t="b">
         <v>0</v>
@@ -56972,65 +56996,65 @@
       </c>
       <c r="P320" t="inlineStr">
         <is>
-          <t>Rafael Silva Alves de Oliveira</t>
+          <t>Guilherme Campos De Arruda Lamego</t>
         </is>
       </c>
       <c r="Q320" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="R320" t="inlineStr">
         <is>
-          <t>Gestão</t>
+          <t>Corte</t>
         </is>
       </c>
       <c r="S320" t="inlineStr">
         <is>
-          <t>Curso: Pós Gestão Fazendas Online Turma: 1 Disciplina: Aplicação de ferramentas e métodos de gestão Tópico: Gestão da rotina de trabalho do dia a dia, qualidade, metas e rituais de gestão Professor: Rafael Silva Alves de OliveiraTipo de Conteúdo: Onli</t>
+          <t>Curso: Pós Corte Online Turma: 21 Disciplina: Princípios da gestão eficiente Tópico: Gestão economico-financeira em fazendas Professor: Guilherme Campos De Arruda LamegoData: 45980</t>
         </is>
       </c>
       <c r="T320" t="inlineStr">
         <is>
-          <t>Pós Gestão Fazendas Online</t>
+          <t>Pós Corte Online</t>
         </is>
       </c>
       <c r="U320" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>21</t>
         </is>
       </c>
       <c r="V320" t="inlineStr">
         <is>
-          <t>Aplicação de ferramentas e métodos de gestão</t>
+          <t>Princípios da gestão eficiente</t>
         </is>
       </c>
       <c r="W320" t="inlineStr">
         <is>
-          <t>Gestão da rotina de trabalho do dia a dia, qualidade, metas e rituais de gestão</t>
+          <t>Gestão economico-financeira em fazendas</t>
         </is>
       </c>
       <c r="X320" s="2">
-        <v>46077.87559027778</v>
+        <v>45979.875</v>
       </c>
       <c r="Y320" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2025-10-29</t>
         </is>
       </c>
       <c r="Z320" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2025-11-05</t>
         </is>
       </c>
       <c r="AA320" t="inlineStr">
         <is>
-          <t>https://rehagro.instructure.com/courses/2974</t>
+          <t>https://rehagro.instructure.com/courses/2941/modules</t>
         </is>
       </c>
       <c r="AB320" t="inlineStr">
         <is>
-          <t>https://docs.google.com/document/d/1ERSO1B7ZDvm0nQO6fx1fC6rTnKmNWXqnuUCTRdqjYbc/edit?tab=t.a7jzuflcbwlc</t>
+          <t>https://docs.google.com/document/d/1xcQZxZVIuqxticMYNr2yoDazsNBgfX4BPdfry9LsfBo/edit?tab=t.19lbzndilb0h</t>
         </is>
       </c>
       <c r="AC320" t="inlineStr">
@@ -57050,58 +57074,58 @@
       </c>
       <c r="AF320" t="inlineStr">
         <is>
-          <t>Gestão</t>
+          <t>Reprovado na Validação</t>
         </is>
       </c>
       <c r="AG320" t="inlineStr">
         <is>
-          <t>01:49:00</t>
+          <t>01:47:00</t>
         </is>
       </c>
       <c r="AH320">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="AI320" s="2">
-        <v>46050.61468837963</v>
+        <v>45908.53444015046</v>
       </c>
       <c r="AJ320" s="2">
-        <v>46072.42328466436</v>
+        <v>45947.59307728009</v>
       </c>
       <c r="AK320">
-        <v>21.808588</v>
+        <v>39.058634</v>
       </c>
       <c r="AL320" s="2">
-        <v>46072.42328561343</v>
+        <v>45947.59307776621</v>
       </c>
       <c r="AM320" s="2">
-        <v>46076.34390538195</v>
+        <v>45952.56312944445</v>
       </c>
       <c r="AN320">
-        <v>3.920613</v>
+        <v>1.110625</v>
       </c>
       <c r="AO320" s="2">
-        <v>46076.34390559028</v>
+        <v>45947.59427358797</v>
       </c>
       <c r="AP320" s="2">
-        <v>46077.68847505787</v>
+        <v>45952.67415577546</v>
       </c>
       <c r="AQ320">
-        <v>1.34456</v>
+        <v>3.97044</v>
       </c>
       <c r="AR320" s="2">
-        <v>46077.68847538195</v>
+        <v>45952.67415603009</v>
       </c>
       <c r="AS320" s="2">
-        <v>46077.70090915509</v>
+        <v>45954.62754299769</v>
       </c>
       <c r="AT320">
-        <v>0.012431</v>
+        <v>1.95338</v>
       </c>
       <c r="AU320" s="2">
-        <v>46077.70090952546</v>
+        <v>45954.62754329861</v>
       </c>
       <c r="AW320">
-        <v>13.571042</v>
+        <v>137.64441</v>
       </c>
     </row>
     <row r="321" ht="18" customHeight="1">
@@ -57235,7 +57259,7 @@
         <v>46090.58107568287</v>
       </c>
       <c r="AQ321">
-        <v>0.69088</v>
+        <v>1.69088</v>
       </c>
     </row>
     <row r="322" ht="18" customHeight="1">
@@ -57249,7 +57273,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Validação</t>
+          <t>Publicar na plataforma</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -57269,7 +57293,7 @@
         <v>46045.58499030092</v>
       </c>
       <c r="J322" s="2">
-        <v>46090.72972653935</v>
+        <v>46091.62671137732</v>
       </c>
       <c r="M322" s="2">
         <v>46075.58499030092</v>
@@ -57345,6 +57369,21 @@
           <t>https://docs.google.com/document/d/1ERSO1B7ZDvm0nQO6fx1fC6rTnKmNWXqnuUCTRdqjYbc/edit?tab=t.aspbfo3qvjqw</t>
         </is>
       </c>
+      <c r="AC322" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="AD322" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="AE322" t="inlineStr">
+        <is>
+          <t>Aprovado: Publicar !</t>
+        </is>
+      </c>
       <c r="AF322" t="inlineStr">
         <is>
           <t>Gestão</t>
@@ -57371,8 +57410,17 @@
       <c r="AO322" s="2">
         <v>46090.72972311343</v>
       </c>
+      <c r="AP322" s="2">
+        <v>46091.62671181713</v>
+      </c>
       <c r="AQ322">
-        <v>0.542222</v>
+        <v>0.896979</v>
+      </c>
+      <c r="AR322" s="2">
+        <v>46091.62671216435</v>
+      </c>
+      <c r="AT322">
+        <v>0.645243</v>
       </c>
     </row>
     <row r="323" ht="18" customHeight="1">
@@ -57553,7 +57601,7 @@
         <v>45873.70610516204</v>
       </c>
       <c r="AW323">
-        <v>217.566829</v>
+        <v>218.566829</v>
       </c>
     </row>
     <row r="324" ht="18" customHeight="1">
@@ -57734,7 +57782,7 @@
         <v>45840.40468760417</v>
       </c>
       <c r="AW324">
-        <v>230.872072</v>
+        <v>231.872072</v>
       </c>
     </row>
     <row r="325" ht="18" customHeight="1">
@@ -57912,7 +57960,7 @@
         <v>46051.66997212963</v>
       </c>
       <c r="AW325">
-        <v>39.601979</v>
+        <v>40.601979</v>
       </c>
     </row>
     <row r="326" ht="18" customHeight="1">
@@ -58090,7 +58138,7 @@
         <v>45817.43653768519</v>
       </c>
       <c r="AW326">
-        <v>273.835417</v>
+        <v>274.835417</v>
       </c>
     </row>
     <row r="327" ht="18" customHeight="1">
@@ -58271,7 +58319,7 @@
         <v>45923.32032945602</v>
       </c>
       <c r="AW327">
-        <v>167.95162</v>
+        <v>168.95162</v>
       </c>
     </row>
     <row r="328" ht="18" customHeight="1">
@@ -58449,7 +58497,7 @@
         <v>45959.61025383102</v>
       </c>
       <c r="AW328">
-        <v>131.661701</v>
+        <v>132.661701</v>
       </c>
     </row>
     <row r="329" ht="18" customHeight="1">
@@ -58630,7 +58678,7 @@
         <v>45971.57499085648</v>
       </c>
       <c r="AW329">
-        <v>119.696956</v>
+        <v>120.696956</v>
       </c>
     </row>
     <row r="330" ht="18" customHeight="1">
@@ -58811,7 +58859,7 @@
         <v>45838.66248615741</v>
       </c>
       <c r="AW330">
-        <v>252.609468</v>
+        <v>253.609468</v>
       </c>
     </row>
     <row r="331" ht="18" customHeight="1">
@@ -58992,7 +59040,7 @@
         <v>45883.60346527777</v>
       </c>
       <c r="AW331">
-        <v>207.668484</v>
+        <v>208.668484</v>
       </c>
     </row>
     <row r="332" ht="18" customHeight="1">
@@ -59173,7 +59221,7 @@
         <v>46001.4599725</v>
       </c>
       <c r="AW332">
-        <v>89.81197899999999</v>
+        <v>90.81197899999999</v>
       </c>
     </row>
     <row r="333" ht="18" customHeight="1">
@@ -59354,7 +59402,7 @@
         <v>46042.45735565972</v>
       </c>
       <c r="AW333">
-        <v>48.814595</v>
+        <v>49.814595</v>
       </c>
     </row>
     <row r="334" ht="18" customHeight="1">
@@ -59532,7 +59580,7 @@
         <v>45890.69609947917</v>
       </c>
       <c r="AW334">
-        <v>200.575856</v>
+        <v>201.575856</v>
       </c>
     </row>
     <row r="335" ht="18" customHeight="1">
@@ -59716,7 +59764,7 @@
         <v>45944.68359482639</v>
       </c>
       <c r="AW335">
-        <v>146.586574</v>
+        <v>147.586574</v>
       </c>
     </row>
     <row r="336" ht="18" customHeight="1">
@@ -59894,7 +59942,7 @@
         <v>45859.70298075231</v>
       </c>
       <c r="AW336">
-        <v>231.56897</v>
+        <v>232.56897</v>
       </c>
     </row>
     <row r="337" ht="18" customHeight="1">
@@ -60075,7 +60123,7 @@
         <v>45965.38240310185</v>
       </c>
       <c r="AW337">
-        <v>125.889549</v>
+        <v>126.889549</v>
       </c>
     </row>
     <row r="338" ht="18" customHeight="1">
@@ -60256,7 +60304,7 @@
         <v>45975.64912039351</v>
       </c>
       <c r="AW338">
-        <v>115.622824</v>
+        <v>116.622824</v>
       </c>
     </row>
     <row r="339" ht="18" customHeight="1">
@@ -60434,7 +60482,7 @@
         <v>45880.67850293982</v>
       </c>
       <c r="AW339">
-        <v>210.593449</v>
+        <v>211.593449</v>
       </c>
     </row>
     <row r="340" ht="18" customHeight="1">
@@ -60615,7 +60663,7 @@
         <v>46034.69664187499</v>
       </c>
       <c r="AW340">
-        <v>56.575313</v>
+        <v>57.575313</v>
       </c>
     </row>
     <row r="341" ht="18" customHeight="1">
@@ -60796,7 +60844,7 @@
         <v>45888.44706435185</v>
       </c>
       <c r="AW341">
-        <v>202.824884</v>
+        <v>203.824884</v>
       </c>
     </row>
     <row r="342" ht="18" customHeight="1">
@@ -60972,7 +61020,7 @@
         <v>45954.62802541666</v>
       </c>
       <c r="AW342">
-        <v>136.643924</v>
+        <v>137.643924</v>
       </c>
     </row>
     <row r="343" ht="18" customHeight="1">
@@ -61073,7 +61121,7 @@
         <v>46076.60422097222</v>
       </c>
       <c r="AK343">
-        <v>14.667731</v>
+        <v>15.667731</v>
       </c>
     </row>
     <row r="344" ht="18" customHeight="1">
@@ -61113,7 +61161,7 @@
         <v>46080.60364699074</v>
       </c>
       <c r="N344" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O344" t="inlineStr">
         <is>
@@ -61210,7 +61258,7 @@
         <v>46079.38060059027</v>
       </c>
       <c r="AQ344">
-        <v>11.891354</v>
+        <v>12.891354</v>
       </c>
     </row>
     <row r="345" ht="18" customHeight="1">
@@ -61388,7 +61436,7 @@
         <v>45812.5781485301</v>
       </c>
       <c r="AW345">
-        <v>278.693796</v>
+        <v>279.693796</v>
       </c>
     </row>
     <row r="346" ht="18" customHeight="1">
@@ -61569,7 +61617,7 @@
         <v>45902.37917880787</v>
       </c>
       <c r="AW346">
-        <v>188.892766</v>
+        <v>189.892766</v>
       </c>
     </row>
     <row r="347" ht="18" customHeight="1">
@@ -61750,7 +61798,7 @@
         <v>45923.31296491898</v>
       </c>
       <c r="AW347">
-        <v>167.958981</v>
+        <v>168.958981</v>
       </c>
     </row>
     <row r="348" ht="18" customHeight="1">
@@ -61931,7 +61979,7 @@
         <v>45973.66494252314</v>
       </c>
       <c r="AW348">
-        <v>117.607002</v>
+        <v>118.607002</v>
       </c>
     </row>
     <row r="349" ht="18" customHeight="1">
@@ -62112,7 +62160,7 @@
         <v>45855.33980681713</v>
       </c>
       <c r="AW349">
-        <v>235.932141</v>
+        <v>236.932141</v>
       </c>
     </row>
     <row r="350" ht="18" customHeight="1">
@@ -62293,7 +62341,7 @@
         <v>46057.49907950232</v>
       </c>
       <c r="AW350">
-        <v>33.77287</v>
+        <v>34.77287</v>
       </c>
     </row>
     <row r="351" ht="18" customHeight="1">
@@ -62474,7 +62522,7 @@
         <v>46076.32663673611</v>
       </c>
       <c r="AW351">
-        <v>14.945313</v>
+        <v>15.945313</v>
       </c>
     </row>
     <row r="352" ht="18" customHeight="1">
@@ -62655,7 +62703,7 @@
         <v>45992.61622836806</v>
       </c>
       <c r="AW352">
-        <v>98.65571799999999</v>
+        <v>99.65571799999999</v>
       </c>
     </row>
     <row r="353" ht="18" customHeight="1">
@@ -62833,7 +62881,7 @@
         <v>45898.61942834491</v>
       </c>
       <c r="AW353">
-        <v>192.652523</v>
+        <v>193.652523</v>
       </c>
     </row>
     <row r="354" ht="18" customHeight="1">
@@ -63014,7 +63062,7 @@
         <v>45919.68091108797</v>
       </c>
       <c r="AW354">
-        <v>171.591042</v>
+        <v>172.591042</v>
       </c>
     </row>
     <row r="355" ht="18" customHeight="1">
@@ -63192,7 +63240,7 @@
         <v>45954.62691407408</v>
       </c>
       <c r="AW355">
-        <v>136.645035</v>
+        <v>137.645035</v>
       </c>
     </row>
     <row r="356" ht="18" customHeight="1">
@@ -63373,7 +63421,7 @@
         <v>45973.66372342593</v>
       </c>
       <c r="AW356">
-        <v>117.608229</v>
+        <v>118.608229</v>
       </c>
     </row>
     <row r="357" ht="18" customHeight="1">
@@ -63554,7 +63602,7 @@
         <v>45846.35986268519</v>
       </c>
       <c r="AW357">
-        <v>244.912083</v>
+        <v>245.912083</v>
       </c>
     </row>
     <row r="358" ht="18" customHeight="1">
@@ -63735,7 +63783,7 @@
         <v>45917.46567336806</v>
       </c>
       <c r="AW358">
-        <v>173.806273</v>
+        <v>174.806273</v>
       </c>
     </row>
     <row r="359" ht="18" customHeight="1">
@@ -63916,7 +63964,7 @@
         <v>45929.33197420138</v>
       </c>
       <c r="AW359">
-        <v>161.939977</v>
+        <v>162.939977</v>
       </c>
     </row>
     <row r="360" ht="18" customHeight="1">
@@ -64097,7 +64145,7 @@
         <v>45915.4691385301</v>
       </c>
       <c r="AW360">
-        <v>168.012488</v>
+        <v>169.012488</v>
       </c>
     </row>
     <row r="361" ht="18" customHeight="1">
@@ -64278,7 +64326,7 @@
         <v>45987.54471672454</v>
       </c>
       <c r="AW361">
-        <v>103.727234</v>
+        <v>104.727234</v>
       </c>
     </row>
     <row r="362" ht="18" customHeight="1">
@@ -64459,7 +64507,7 @@
         <v>46037.66552774305</v>
       </c>
       <c r="AW362">
-        <v>53.606424</v>
+        <v>54.606424</v>
       </c>
     </row>
     <row r="363" ht="18" customHeight="1">
@@ -64640,7 +64688,7 @@
         <v>45821.67524549768</v>
       </c>
       <c r="AW363">
-        <v>269.596701</v>
+        <v>270.596701</v>
       </c>
     </row>
     <row r="364" ht="18" customHeight="1">
@@ -64818,7 +64866,7 @@
         <v>45820.3330696875</v>
       </c>
       <c r="AW364">
-        <v>270.938877</v>
+        <v>271.938877</v>
       </c>
     </row>
     <row r="365" ht="18" customHeight="1">
@@ -64999,7 +65047,7 @@
         <v>46006.54578523149</v>
       </c>
       <c r="AW365">
-        <v>84.726169</v>
+        <v>85.726169</v>
       </c>
     </row>
     <row r="366" ht="18" customHeight="1">
@@ -65180,7 +65228,7 @@
         <v>46051.53146484954</v>
       </c>
       <c r="AW366">
-        <v>39.740486</v>
+        <v>40.740486</v>
       </c>
     </row>
     <row r="367" ht="18" customHeight="1">
@@ -65358,7 +65406,7 @@
         <v>45813.68440848379</v>
       </c>
       <c r="AW367">
-        <v>277.587546</v>
+        <v>278.587546</v>
       </c>
     </row>
     <row r="368" ht="18" customHeight="1">
@@ -65539,7 +65587,7 @@
         <v>45923.31175675926</v>
       </c>
       <c r="AW368">
-        <v>167.960197</v>
+        <v>168.960197</v>
       </c>
     </row>
     <row r="369" ht="18" customHeight="1">
@@ -65717,7 +65765,7 @@
         <v>46003.56407180555</v>
       </c>
       <c r="AW369">
-        <v>87.707882</v>
+        <v>88.707882</v>
       </c>
     </row>
     <row r="370" ht="18" customHeight="1">
@@ -65898,7 +65946,7 @@
         <v>45842.70903693287</v>
       </c>
       <c r="AW370">
-        <v>248.562917</v>
+        <v>249.562917</v>
       </c>
     </row>
     <row r="371" ht="18" customHeight="1">
@@ -66079,7 +66127,7 @@
         <v>45952.41448010417</v>
       </c>
       <c r="AW371">
-        <v>138.857465</v>
+        <v>139.857465</v>
       </c>
     </row>
     <row r="372" ht="18" customHeight="1">
@@ -66260,7 +66308,7 @@
         <v>45954.37944618055</v>
       </c>
       <c r="AW372">
-        <v>136.8925</v>
+        <v>137.8925</v>
       </c>
     </row>
     <row r="373" ht="18" customHeight="1">
@@ -66438,7 +66486,7 @@
         <v>45826.77024422454</v>
       </c>
       <c r="AW373">
-        <v>264.501701</v>
+        <v>265.501701</v>
       </c>
     </row>
     <row r="374" ht="18" customHeight="1">
@@ -66619,7 +66667,7 @@
         <v>45855.34249084491</v>
       </c>
       <c r="AW374">
-        <v>235.929456</v>
+        <v>236.929456</v>
       </c>
     </row>
     <row r="375" ht="18" customHeight="1">
@@ -66797,7 +66845,7 @@
         <v>45936.74229829861</v>
       </c>
       <c r="AW375">
-        <v>154.529653</v>
+        <v>155.529653</v>
       </c>
     </row>
     <row r="376" ht="18" customHeight="1">
@@ -66913,7 +66961,7 @@
         <v>46077.71026703704</v>
       </c>
       <c r="AN376">
-        <v>11.610671</v>
+        <v>12.610671</v>
       </c>
     </row>
     <row r="377" ht="18" customHeight="1">
@@ -67091,7 +67139,7 @@
         <v>45852.54993511573</v>
       </c>
       <c r="AW377">
-        <v>238.722014</v>
+        <v>239.722014</v>
       </c>
     </row>
     <row r="378" ht="18" customHeight="1">
@@ -67272,7 +67320,7 @@
         <v>45904.38291060185</v>
       </c>
       <c r="AW378">
-        <v>186.889039</v>
+        <v>187.889039</v>
       </c>
     </row>
     <row r="379" ht="18" customHeight="1">
@@ -67306,13 +67354,13 @@
         <v>46045.58497321759</v>
       </c>
       <c r="J379" s="2">
-        <v>46090.40562921297</v>
+        <v>46091.40575797453</v>
       </c>
       <c r="M379" s="2">
         <v>46075.58497321759</v>
       </c>
       <c r="N379" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O379" t="inlineStr">
         <is>
@@ -67433,7 +67481,7 @@
         <v>46090.40563063657</v>
       </c>
       <c r="AT379">
-        <v>0.866319</v>
+        <v>1.866319</v>
       </c>
     </row>
     <row r="380" ht="18" customHeight="1">
@@ -67611,7 +67659,7 @@
         <v>45810.36123126157</v>
       </c>
       <c r="AW380">
-        <v>273.727454</v>
+        <v>274.727454</v>
       </c>
     </row>
     <row r="381" ht="18" customHeight="1">
@@ -67789,7 +67837,7 @@
         <v>45821.63864346065</v>
       </c>
       <c r="AW381">
-        <v>269.63331</v>
+        <v>270.63331</v>
       </c>
     </row>
     <row r="382" ht="18" customHeight="1">
@@ -67970,7 +68018,7 @@
         <v>45973.65832961806</v>
       </c>
       <c r="AW382">
-        <v>117.613623</v>
+        <v>118.613623</v>
       </c>
     </row>
     <row r="383" ht="18" customHeight="1">
@@ -68148,7 +68196,7 @@
         <v>45820.3322787037</v>
       </c>
       <c r="AW383">
-        <v>270.939676</v>
+        <v>271.939676</v>
       </c>
     </row>
     <row r="384" ht="18" customHeight="1">
@@ -68326,7 +68374,7 @@
         <v>45842.70851819444</v>
       </c>
       <c r="AW384">
-        <v>248.563438</v>
+        <v>249.563438</v>
       </c>
     </row>
     <row r="385" ht="18" customHeight="1">
@@ -68504,7 +68552,7 @@
         <v>45812.58675498843</v>
       </c>
       <c r="AW385">
-        <v>278.685197</v>
+        <v>279.685197</v>
       </c>
     </row>
     <row r="386" ht="18" customHeight="1">
@@ -68682,7 +68730,7 @@
         <v>45964.65037627315</v>
       </c>
       <c r="AW386">
-        <v>126.621574</v>
+        <v>127.621574</v>
       </c>
     </row>
     <row r="387" ht="18" customHeight="1">
@@ -68860,7 +68908,7 @@
         <v>45826.77171652778</v>
       </c>
       <c r="AW387">
-        <v>264.500231</v>
+        <v>265.500231</v>
       </c>
     </row>
     <row r="388" ht="18" customHeight="1">
@@ -69038,7 +69086,7 @@
         <v>45859.70584207177</v>
       </c>
       <c r="AW388">
-        <v>231.566111</v>
+        <v>232.566111</v>
       </c>
     </row>
     <row r="389" ht="18" customHeight="1">
@@ -69219,7 +69267,7 @@
         <v>45868.57320862269</v>
       </c>
       <c r="AW389">
-        <v>222.698738</v>
+        <v>223.698738</v>
       </c>
     </row>
     <row r="390" ht="18" customHeight="1">
@@ -69400,7 +69448,7 @@
         <v>45952.41516831018</v>
       </c>
       <c r="AW390">
-        <v>138.856782</v>
+        <v>139.856782</v>
       </c>
     </row>
     <row r="391" ht="18" customHeight="1">
@@ -69581,7 +69629,7 @@
         <v>46007.42823478009</v>
       </c>
       <c r="AW391">
-        <v>83.843715</v>
+        <v>84.843715</v>
       </c>
     </row>
     <row r="392" ht="18" customHeight="1">
@@ -69762,7 +69810,7 @@
         <v>46001.46105103009</v>
       </c>
       <c r="AW392">
-        <v>89.810903</v>
+        <v>90.810903</v>
       </c>
     </row>
     <row r="393" ht="18" customHeight="1">
@@ -69935,7 +69983,7 @@
         <v>45905.67968340278</v>
       </c>
       <c r="AW393">
-        <v>185.592269</v>
+        <v>186.592269</v>
       </c>
     </row>
     <row r="394" ht="18" customHeight="1">
@@ -70108,7 +70156,7 @@
         <v>45905.68014417824</v>
       </c>
       <c r="AW394">
-        <v>185.591806</v>
+        <v>186.591806</v>
       </c>
     </row>
     <row r="395" ht="18" customHeight="1">
@@ -70289,7 +70337,7 @@
         <v>46001.46262186342</v>
       </c>
       <c r="AW395">
-        <v>89.80932900000001</v>
+        <v>90.80932900000001</v>
       </c>
     </row>
     <row r="396" ht="18" customHeight="1">
@@ -70470,7 +70518,7 @@
         <v>45986.56209506944</v>
       </c>
       <c r="AW396">
-        <v>104.70985</v>
+        <v>105.70985</v>
       </c>
     </row>
     <row r="397" ht="18" customHeight="1">
@@ -70651,7 +70699,7 @@
         <v>45973.66474306713</v>
       </c>
       <c r="AW397">
-        <v>117.607211</v>
+        <v>118.607211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>